<commit_message>
Validation and packages book 3
</commit_message>
<xml_diff>
--- a/data/Influencers_OLS.xlsx
+++ b/data/Influencers_OLS.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,102 +441,102 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>565</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>871</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>351</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>725</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>871</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>584</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>375</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>471</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>214</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>351</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>549</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>863</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>678</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>625</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>526</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>863</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>526</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>584</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>712</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>625</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>864</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>678</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>565</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>334</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>549</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>375</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>471</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>229</t>
         </is>
       </c>
     </row>
@@ -574,31 +574,31 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
         <v>0.1508</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
       </c>
       <c r="T2" t="n">
         <v>0</v>
@@ -638,10 +638,10 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>2.42</v>
       </c>
       <c r="I3" t="n">
-        <v>2.42</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -656,7 +656,7 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>2.48</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -668,7 +668,7 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>2.48</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
         <v>0</v>
@@ -705,47 +705,47 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.0767</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>5.8839</v>
+      </c>
+      <c r="M4" t="n">
         <v>0.921</v>
       </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
+      <c r="N4" t="n">
+        <v>0.2047</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
         <v>0.0767</v>
       </c>
-      <c r="L4" t="n">
-        <v>0.0767</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0.2047</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0</v>
-      </c>
       <c r="T4" t="n">
         <v>0</v>
       </c>
@@ -753,10 +753,10 @@
         <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>5.8839</v>
+        <v>11.9724</v>
       </c>
       <c r="W4" t="n">
-        <v>11.9724</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -778,47 +778,47 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.1188</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1.1592</v>
+      </c>
+      <c r="M5" t="n">
         <v>0.3021</v>
       </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
+      <c r="N5" t="n">
+        <v>0.07489999999999999</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
         <v>0.0336</v>
       </c>
-      <c r="L5" t="n">
-        <v>0.1188</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" t="n">
-        <v>0.07489999999999999</v>
-      </c>
-      <c r="S5" t="n">
-        <v>0</v>
-      </c>
       <c r="T5" t="n">
         <v>0</v>
       </c>
@@ -826,10 +826,10 @@
         <v>0</v>
       </c>
       <c r="V5" t="n">
-        <v>1.1592</v>
+        <v>0.1394</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1394</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -851,31 +851,31 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.0595</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.5558</v>
+      </c>
+      <c r="M6" t="n">
         <v>0.6947</v>
       </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.0595</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>3.156</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -887,7 +887,7 @@
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>3.156</v>
+        <v>0</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
@@ -899,10 +899,10 @@
         <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>0.5558</v>
+        <v>0.8535</v>
       </c>
       <c r="W6" t="n">
-        <v>0.8535</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -924,47 +924,47 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.0504</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.1512</v>
+      </c>
+      <c r="M7" t="n">
         <v>13.5058</v>
       </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
+      <c r="N7" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
         <v>1.2431</v>
       </c>
-      <c r="L7" t="n">
-        <v>0.0504</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0.168</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0</v>
-      </c>
       <c r="T7" t="n">
         <v>0</v>
       </c>
@@ -972,10 +972,10 @@
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>0.1512</v>
+        <v>4.9051</v>
       </c>
       <c r="W7" t="n">
-        <v>4.9051</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -997,47 +997,47 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2.3622</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.3656</v>
+      </c>
+      <c r="M8" t="n">
         <v>3.6515</v>
       </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
+      <c r="N8" t="n">
+        <v>0.3127</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
         <v>1.2749</v>
       </c>
-      <c r="L8" t="n">
-        <v>2.3622</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0.3127</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0</v>
-      </c>
       <c r="T8" t="n">
         <v>0</v>
       </c>
@@ -1045,10 +1045,10 @@
         <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>0.3656</v>
+        <v>2.7326</v>
       </c>
       <c r="W8" t="n">
-        <v>2.7326</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1070,47 +1070,47 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.08550000000000001</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.2541</v>
+      </c>
+      <c r="M9" t="n">
         <v>0.9429999999999999</v>
       </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
+      <c r="N9" t="n">
+        <v>3.4666</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" t="n">
         <v>0.1686</v>
       </c>
-      <c r="L9" t="n">
-        <v>0.08550000000000001</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" t="n">
-        <v>3.4666</v>
-      </c>
-      <c r="S9" t="n">
-        <v>0</v>
-      </c>
       <c r="T9" t="n">
         <v>0</v>
       </c>
@@ -1118,10 +1118,10 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>0.2541</v>
+        <v>0.9258999999999999</v>
       </c>
       <c r="W9" t="n">
-        <v>0.9258999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1170,25 +1170,25 @@
         <v>0</v>
       </c>
       <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" t="n">
         <v>0.1059</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U10" t="n">
-        <v>0</v>
       </c>
       <c r="V10" t="n">
         <v>0</v>
@@ -1210,64 +1210,64 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
+        <v>0.2643</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.4404</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1.8498</v>
+      </c>
+      <c r="I11" t="n">
         <v>0.1762</v>
       </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.4404</v>
-      </c>
-      <c r="H11" t="n">
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.7927999999999999</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>2.7054</v>
+      </c>
+      <c r="P11" t="n">
+        <v>1.661</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.0126</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0.0126</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" t="n">
         <v>0.151</v>
       </c>
-      <c r="I11" t="n">
-        <v>1.8498</v>
-      </c>
-      <c r="J11" t="n">
-        <v>1.661</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" t="n">
+      <c r="U11" t="n">
+        <v>0.2517</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" t="n">
         <v>0.0126</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0.2517</v>
-      </c>
-      <c r="P11" t="n">
-        <v>0.0126</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0.2643</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0.0126</v>
-      </c>
-      <c r="T11" t="n">
-        <v>2.7054</v>
-      </c>
-      <c r="U11" t="n">
-        <v>0.7927999999999999</v>
-      </c>
-      <c r="V11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W11" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1337,10 +1337,10 @@
         <v>0</v>
       </c>
       <c r="V12" t="n">
-        <v>0</v>
+        <v>0.0029</v>
       </c>
       <c r="W12" t="n">
-        <v>0.0029</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1356,58 +1356,58 @@
         <v>1</v>
       </c>
       <c r="D13" t="n">
+        <v>0.2466</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.6261</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.1138</v>
+      </c>
+      <c r="I13" t="n">
         <v>0.3035</v>
       </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.6261</v>
-      </c>
-      <c r="H13" t="n">
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.702</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.3035</v>
+      </c>
+      <c r="P13" t="n">
+        <v>2.1628</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" t="n">
         <v>1.2332</v>
       </c>
-      <c r="I13" t="n">
-        <v>0.1138</v>
-      </c>
-      <c r="J13" t="n">
-        <v>2.1628</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" t="n">
+      <c r="U13" t="n">
         <v>3.2821</v>
-      </c>
-      <c r="P13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0.2466</v>
-      </c>
-      <c r="R13" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" t="n">
-        <v>0.3035</v>
-      </c>
-      <c r="U13" t="n">
-        <v>0.702</v>
       </c>
       <c r="V13" t="n">
         <v>0</v>
@@ -1441,10 +1441,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>0.0144</v>
       </c>
       <c r="I14" t="n">
-        <v>0.0144</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -1520,31 +1520,31 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
         <v>0.0047</v>
       </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" t="n">
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="n">
         <v>0.295</v>
-      </c>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0</v>
       </c>
       <c r="S15" t="n">
         <v>0</v>
@@ -1581,47 +1581,47 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.1326</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.7877</v>
+      </c>
+      <c r="M16" t="n">
         <v>1.3715</v>
       </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
+      <c r="N16" t="n">
+        <v>0.4334</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="n">
         <v>0.0867</v>
       </c>
-      <c r="L16" t="n">
-        <v>0.1326</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" t="n">
-        <v>0.4334</v>
-      </c>
-      <c r="S16" t="n">
-        <v>0</v>
-      </c>
       <c r="T16" t="n">
         <v>0</v>
       </c>
@@ -1629,10 +1629,10 @@
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>0.7877</v>
+        <v>0.8999</v>
       </c>
       <c r="W16" t="n">
-        <v>0.8999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -1654,31 +1654,31 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
         <v>3.2514</v>
       </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0</v>
-      </c>
       <c r="N17" t="n">
-        <v>0</v>
+        <v>0.3597</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
@@ -1690,7 +1690,7 @@
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>0.3597</v>
+        <v>0</v>
       </c>
       <c r="S17" t="n">
         <v>0</v>
@@ -1702,10 +1702,10 @@
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>0</v>
+        <v>2.605</v>
       </c>
       <c r="W17" t="n">
-        <v>2.605</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1721,7 +1721,7 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -1733,52 +1733,52 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
+        <v>0.0944</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" t="n">
         <v>0.005</v>
       </c>
-      <c r="I18" t="n">
-        <v>0.0944</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0.0298</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" t="n">
+      <c r="S18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" t="n">
         <v>0.005</v>
       </c>
-      <c r="O18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="R18" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" t="n">
+      <c r="U18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" t="n">
+        <v>0</v>
+      </c>
+      <c r="W18" t="n">
         <v>0.009900000000000001</v>
-      </c>
-      <c r="T18" t="n">
-        <v>0</v>
-      </c>
-      <c r="U18" t="n">
-        <v>0</v>
-      </c>
-      <c r="V18" t="n">
-        <v>0</v>
-      </c>
-      <c r="W18" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1800,43 +1800,43 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>0.06610000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>0.06610000000000001</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>0.8107</v>
       </c>
       <c r="I19" t="n">
-        <v>0.8107</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.0259</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
         <v>0.3076</v>
       </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" t="n">
-        <v>0</v>
-      </c>
       <c r="Q19" t="n">
         <v>0</v>
       </c>
       <c r="R19" t="n">
-        <v>0.0259</v>
+        <v>0</v>
       </c>
       <c r="S19" t="n">
         <v>0</v>
@@ -1848,10 +1848,10 @@
         <v>0</v>
       </c>
       <c r="V19" t="n">
-        <v>0</v>
+        <v>0.0029</v>
       </c>
       <c r="W19" t="n">
-        <v>0.0029</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1897,25 +1897,25 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.3998</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" t="n">
         <v>0.0013</v>
       </c>
-      <c r="O20" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0</v>
-      </c>
       <c r="S20" t="n">
         <v>0</v>
       </c>
       <c r="T20" t="n">
-        <v>0.3998</v>
+        <v>0</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -1946,10 +1946,10 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>0.0016</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0016</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -2013,64 +2013,64 @@
         <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>0.0078</v>
+        <v>0.0117</v>
       </c>
       <c r="E22" t="n">
         <v>0.4069</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>0.0157</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0157</v>
+        <v>1.4751</v>
       </c>
       <c r="H22" t="n">
+        <v>5.1571</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.0078</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.1683</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" t="n">
+        <v>7.1605</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0.2191</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>1.4986</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0.4617</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" t="n">
         <v>0.0391</v>
       </c>
-      <c r="I22" t="n">
-        <v>5.1571</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0.2191</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" t="n">
-        <v>1.4751</v>
-      </c>
-      <c r="N22" t="n">
-        <v>0.4617</v>
-      </c>
-      <c r="O22" t="n">
+      <c r="U22" t="n">
         <v>0.043</v>
       </c>
-      <c r="P22" t="n">
-        <v>1.4986</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>0.0117</v>
-      </c>
-      <c r="R22" t="n">
-        <v>0</v>
-      </c>
-      <c r="S22" t="n">
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W22" t="n">
         <v>1.7373</v>
-      </c>
-      <c r="T22" t="n">
-        <v>7.1605</v>
-      </c>
-      <c r="U22" t="n">
-        <v>0.1683</v>
-      </c>
-      <c r="V22" t="n">
-        <v>0</v>
-      </c>
-      <c r="W22" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -2092,47 +2092,47 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1.8231</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.1343</v>
+      </c>
+      <c r="M23" t="n">
         <v>0.1151</v>
       </c>
-      <c r="G23" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="n">
+      <c r="N23" t="n">
+        <v>0.2687</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" t="n">
         <v>0.0192</v>
       </c>
-      <c r="L23" t="n">
-        <v>1.8231</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" t="n">
-        <v>0.2687</v>
-      </c>
-      <c r="S23" t="n">
-        <v>0</v>
-      </c>
       <c r="T23" t="n">
         <v>0</v>
       </c>
@@ -2140,10 +2140,10 @@
         <v>0</v>
       </c>
       <c r="V23" t="n">
-        <v>0.1343</v>
+        <v>0.5757</v>
       </c>
       <c r="W23" t="n">
-        <v>0.5757</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -2159,46 +2159,46 @@
         <v>1</v>
       </c>
       <c r="D24" t="n">
+        <v>1.4854</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.4297</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.0123</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.2332</v>
+      </c>
+      <c r="I24" t="n">
         <v>3.5846</v>
       </c>
-      <c r="E24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0.4297</v>
-      </c>
-      <c r="H24" t="n">
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0.6875</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="n">
         <v>0.3069</v>
       </c>
-      <c r="I24" t="n">
-        <v>0.2332</v>
-      </c>
-      <c r="J24" t="n">
+      <c r="P24" t="n">
         <v>0.8102</v>
       </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0.0123</v>
-      </c>
-      <c r="N24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0.2946</v>
-      </c>
-      <c r="P24" t="n">
-        <v>0</v>
-      </c>
       <c r="Q24" t="n">
-        <v>1.4854</v>
+        <v>0</v>
       </c>
       <c r="R24" t="n">
         <v>0</v>
@@ -2210,7 +2210,7 @@
         <v>0.3069</v>
       </c>
       <c r="U24" t="n">
-        <v>0.6875</v>
+        <v>0.2946</v>
       </c>
       <c r="V24" t="n">
         <v>0</v>
@@ -2238,31 +2238,31 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
+        <v>0.7262999999999999</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="n">
         <v>0.1928</v>
       </c>
-      <c r="G25" t="n">
-        <v>0.7262999999999999</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0</v>
-      </c>
       <c r="N25" t="n">
-        <v>0</v>
+        <v>0.1704</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
@@ -2274,7 +2274,7 @@
         <v>0</v>
       </c>
       <c r="R25" t="n">
-        <v>0.1704</v>
+        <v>0</v>
       </c>
       <c r="S25" t="n">
         <v>0</v>
@@ -2286,10 +2286,10 @@
         <v>0</v>
       </c>
       <c r="V25" t="n">
-        <v>0</v>
+        <v>0.1748</v>
       </c>
       <c r="W25" t="n">
-        <v>0.1748</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -2399,17 +2399,17 @@
         <v>0</v>
       </c>
       <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
         <v>0.0395</v>
       </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" t="n">
-        <v>0</v>
-      </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
@@ -2420,11 +2420,11 @@
         <v>0</v>
       </c>
       <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="n">
         <v>0.0395</v>
       </c>
-      <c r="S27" t="n">
-        <v>0</v>
-      </c>
       <c r="T27" t="n">
         <v>0</v>
       </c>
@@ -2432,10 +2432,10 @@
         <v>0</v>
       </c>
       <c r="V27" t="n">
-        <v>0</v>
+        <v>0.06909999999999999</v>
       </c>
       <c r="W27" t="n">
-        <v>0.06909999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -2463,37 +2463,37 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>0.5959</v>
       </c>
       <c r="I28" t="n">
-        <v>0.5959</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0.0271</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
         <v>0.948</v>
       </c>
-      <c r="K28" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" t="n">
-        <v>0</v>
-      </c>
-      <c r="P28" t="n">
-        <v>0</v>
-      </c>
       <c r="Q28" t="n">
         <v>0</v>
       </c>
       <c r="R28" t="n">
-        <v>0.0271</v>
+        <v>0</v>
       </c>
       <c r="S28" t="n">
         <v>0</v>
@@ -2545,32 +2545,32 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S29" t="n">
         <v>3.1</v>
       </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R29" t="n">
-        <v>0</v>
-      </c>
-      <c r="S29" t="n">
-        <v>0</v>
-      </c>
       <c r="T29" t="n">
         <v>0</v>
       </c>
@@ -2578,10 +2578,10 @@
         <v>0</v>
       </c>
       <c r="V29" t="n">
-        <v>0</v>
+        <v>0.55</v>
       </c>
       <c r="W29" t="n">
-        <v>0.55</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -2597,28 +2597,28 @@
         <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>0.2099</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>0.0579</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0579</v>
+        <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>0.0145</v>
       </c>
       <c r="I30" t="n">
-        <v>0.0145</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>0</v>
+        <v>0.5934</v>
       </c>
       <c r="L30" t="n">
         <v>0</v>
@@ -2627,28 +2627,28 @@
         <v>0</v>
       </c>
       <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="n">
+        <v>1.4328</v>
+      </c>
+      <c r="P30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>3.0972</v>
+      </c>
+      <c r="R30" t="n">
         <v>0.0036</v>
       </c>
-      <c r="O30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P30" t="n">
-        <v>3.0972</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>0.2099</v>
-      </c>
-      <c r="R30" t="n">
-        <v>0</v>
-      </c>
       <c r="S30" t="n">
         <v>0</v>
       </c>
       <c r="T30" t="n">
-        <v>1.4328</v>
+        <v>0</v>
       </c>
       <c r="U30" t="n">
-        <v>0.5934</v>
+        <v>0</v>
       </c>
       <c r="V30" t="n">
         <v>0</v>
@@ -2676,43 +2676,43 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="G31" t="n">
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>0.2917</v>
       </c>
       <c r="I31" t="n">
-        <v>0.2917</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0.0511</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
         <v>0.4151</v>
       </c>
-      <c r="K31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" t="n">
-        <v>0</v>
-      </c>
       <c r="Q31" t="n">
         <v>0</v>
       </c>
       <c r="R31" t="n">
-        <v>0.0511</v>
+        <v>0</v>
       </c>
       <c r="S31" t="n">
         <v>0</v>
@@ -2749,43 +2749,43 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="G32" t="n">
-        <v>0.008200000000000001</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>0.1908</v>
       </c>
       <c r="I32" t="n">
-        <v>0.1908</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0.0277</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
         <v>0.8921</v>
       </c>
-      <c r="K32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P32" t="n">
-        <v>0</v>
-      </c>
       <c r="Q32" t="n">
         <v>0</v>
       </c>
       <c r="R32" t="n">
-        <v>0.0277</v>
+        <v>0</v>
       </c>
       <c r="S32" t="n">
         <v>0</v>
@@ -2822,43 +2822,43 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
+        <v>0.0278</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" t="n">
         <v>0.5633</v>
       </c>
-      <c r="G33" t="n">
-        <v>0.0278</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" t="n">
+      <c r="N33" t="n">
+        <v>0.0129</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" t="n">
         <v>0.0107</v>
       </c>
-      <c r="K33" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" t="n">
-        <v>0</v>
-      </c>
-      <c r="M33" t="n">
-        <v>0</v>
-      </c>
-      <c r="N33" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" t="n">
-        <v>0</v>
-      </c>
-      <c r="P33" t="n">
-        <v>0</v>
-      </c>
       <c r="Q33" t="n">
         <v>0</v>
       </c>
       <c r="R33" t="n">
-        <v>0.0129</v>
+        <v>0</v>
       </c>
       <c r="S33" t="n">
         <v>0</v>
@@ -2870,10 +2870,10 @@
         <v>0</v>
       </c>
       <c r="V33" t="n">
-        <v>0</v>
+        <v>0.0493</v>
       </c>
       <c r="W33" t="n">
-        <v>0.0493</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -2895,43 +2895,43 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
+        <v>0.0339</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" t="n">
         <v>0.0774</v>
       </c>
-      <c r="G34" t="n">
-        <v>0.0339</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" t="n">
+      <c r="N34" t="n">
+        <v>0.1065</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" t="n">
         <v>0.0182</v>
       </c>
-      <c r="K34" t="n">
-        <v>0</v>
-      </c>
-      <c r="L34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M34" t="n">
-        <v>0</v>
-      </c>
-      <c r="N34" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" t="n">
-        <v>0</v>
-      </c>
-      <c r="P34" t="n">
-        <v>0</v>
-      </c>
       <c r="Q34" t="n">
         <v>0</v>
       </c>
       <c r="R34" t="n">
-        <v>0.1065</v>
+        <v>0</v>
       </c>
       <c r="S34" t="n">
         <v>0</v>
@@ -2943,10 +2943,10 @@
         <v>0</v>
       </c>
       <c r="V34" t="n">
-        <v>0</v>
+        <v>0.19</v>
       </c>
       <c r="W34" t="n">
-        <v>0.19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -2962,64 +2962,64 @@
         <v>1</v>
       </c>
       <c r="D35" t="n">
+        <v>4.4009</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>5.0709</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.141</v>
+      </c>
+      <c r="I35" t="n">
         <v>2.0539</v>
       </c>
-      <c r="E35" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" t="n">
-        <v>5.0709</v>
-      </c>
-      <c r="H35" t="n">
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0.6016</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0.2292</v>
+      </c>
+      <c r="P35" t="n">
+        <v>1.536</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="S35" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" t="n">
         <v>2.2016</v>
       </c>
-      <c r="I35" t="n">
-        <v>0.141</v>
-      </c>
-      <c r="J35" t="n">
-        <v>1.536</v>
-      </c>
-      <c r="K35" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" t="n">
-        <v>0.0044</v>
-      </c>
-      <c r="O35" t="n">
+      <c r="U35" t="n">
         <v>2.8605</v>
       </c>
-      <c r="P35" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>4.4009</v>
-      </c>
-      <c r="R35" t="n">
-        <v>0</v>
-      </c>
-      <c r="S35" t="n">
+      <c r="V35" t="n">
+        <v>0</v>
+      </c>
+      <c r="W35" t="n">
         <v>0.0022</v>
-      </c>
-      <c r="T35" t="n">
-        <v>0.2292</v>
-      </c>
-      <c r="U35" t="n">
-        <v>0.6016</v>
-      </c>
-      <c r="V35" t="n">
-        <v>0</v>
-      </c>
-      <c r="W35" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -3056,31 +3056,31 @@
         <v>0</v>
       </c>
       <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" t="n">
         <v>1.8556</v>
-      </c>
-      <c r="L36" t="n">
-        <v>0</v>
-      </c>
-      <c r="M36" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" t="n">
-        <v>0</v>
-      </c>
-      <c r="O36" t="n">
-        <v>0</v>
-      </c>
-      <c r="P36" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q36" t="n">
-        <v>0</v>
-      </c>
-      <c r="R36" t="n">
-        <v>0</v>
-      </c>
-      <c r="S36" t="n">
-        <v>0</v>
       </c>
       <c r="T36" t="n">
         <v>0</v>
@@ -3114,37 +3114,37 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>0.0038</v>
       </c>
       <c r="G37" t="n">
-        <v>0.0038</v>
+        <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>0.0075</v>
       </c>
       <c r="I37" t="n">
-        <v>0.0075</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
         <v>0.0263</v>
-      </c>
-      <c r="K37" t="n">
-        <v>0</v>
-      </c>
-      <c r="L37" t="n">
-        <v>0</v>
-      </c>
-      <c r="M37" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" t="n">
-        <v>0</v>
-      </c>
-      <c r="O37" t="n">
-        <v>0</v>
-      </c>
-      <c r="P37" t="n">
-        <v>0</v>
       </c>
       <c r="Q37" t="n">
         <v>0</v>
@@ -3187,31 +3187,31 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" t="n">
         <v>4.2629</v>
       </c>
-      <c r="G38" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="H38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" t="n">
-        <v>0</v>
-      </c>
-      <c r="K38" t="n">
-        <v>0</v>
-      </c>
-      <c r="L38" t="n">
-        <v>0</v>
-      </c>
-      <c r="M38" t="n">
-        <v>0</v>
-      </c>
       <c r="N38" t="n">
-        <v>0</v>
+        <v>0.168</v>
       </c>
       <c r="O38" t="n">
         <v>0</v>
@@ -3223,7 +3223,7 @@
         <v>0</v>
       </c>
       <c r="R38" t="n">
-        <v>0.168</v>
+        <v>0</v>
       </c>
       <c r="S38" t="n">
         <v>0</v>
@@ -3235,10 +3235,10 @@
         <v>0</v>
       </c>
       <c r="V38" t="n">
-        <v>0</v>
+        <v>1.008</v>
       </c>
       <c r="W38" t="n">
-        <v>1.008</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -3260,43 +3260,43 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
+        <v>0.0197</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" t="n">
         <v>0.0493</v>
       </c>
-      <c r="G39" t="n">
-        <v>0.0197</v>
-      </c>
-      <c r="H39" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" t="n">
+      <c r="N39" t="n">
+        <v>0.009900000000000001</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
         <v>0.0985</v>
       </c>
-      <c r="K39" t="n">
-        <v>0</v>
-      </c>
-      <c r="L39" t="n">
-        <v>0</v>
-      </c>
-      <c r="M39" t="n">
-        <v>0</v>
-      </c>
-      <c r="N39" t="n">
-        <v>0</v>
-      </c>
-      <c r="O39" t="n">
-        <v>0</v>
-      </c>
-      <c r="P39" t="n">
-        <v>0</v>
-      </c>
       <c r="Q39" t="n">
         <v>0</v>
       </c>
       <c r="R39" t="n">
-        <v>0.009900000000000001</v>
+        <v>0</v>
       </c>
       <c r="S39" t="n">
         <v>0</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="V39" t="n">
-        <v>0</v>
+        <v>0.1675</v>
       </c>
       <c r="W39" t="n">
-        <v>0.1675</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -3333,28 +3333,28 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" t="n">
         <v>4.41</v>
-      </c>
-      <c r="G40" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" t="n">
-        <v>0</v>
-      </c>
-      <c r="J40" t="n">
-        <v>0</v>
-      </c>
-      <c r="K40" t="n">
-        <v>0</v>
-      </c>
-      <c r="L40" t="n">
-        <v>0</v>
-      </c>
-      <c r="M40" t="n">
-        <v>0</v>
       </c>
       <c r="N40" t="n">
         <v>0</v>
@@ -3406,16 +3406,16 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>6.0048</v>
       </c>
       <c r="G41" t="n">
-        <v>6.0048</v>
+        <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>0.0013</v>
       </c>
       <c r="I41" t="n">
-        <v>0.0013</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -3491,25 +3491,25 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" t="n">
         <v>0.0431</v>
-      </c>
-      <c r="K42" t="n">
-        <v>0</v>
-      </c>
-      <c r="L42" t="n">
-        <v>0</v>
-      </c>
-      <c r="M42" t="n">
-        <v>0</v>
-      </c>
-      <c r="N42" t="n">
-        <v>0</v>
-      </c>
-      <c r="O42" t="n">
-        <v>0</v>
-      </c>
-      <c r="P42" t="n">
-        <v>0</v>
       </c>
       <c r="Q42" t="n">
         <v>0</v>
@@ -3552,47 +3552,47 @@
         <v>0</v>
       </c>
       <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.5569</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0.0497</v>
+      </c>
+      <c r="M43" t="n">
         <v>0.0975</v>
       </c>
-      <c r="G43" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" t="n">
-        <v>0</v>
-      </c>
-      <c r="K43" t="n">
+      <c r="N43" t="n">
+        <v>0.0975</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>0</v>
+      </c>
+      <c r="R43" t="n">
+        <v>0</v>
+      </c>
+      <c r="S43" t="n">
         <v>0.0139</v>
       </c>
-      <c r="L43" t="n">
-        <v>0.5569</v>
-      </c>
-      <c r="M43" t="n">
-        <v>0</v>
-      </c>
-      <c r="N43" t="n">
-        <v>0</v>
-      </c>
-      <c r="O43" t="n">
-        <v>0</v>
-      </c>
-      <c r="P43" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q43" t="n">
-        <v>0</v>
-      </c>
-      <c r="R43" t="n">
-        <v>0.0975</v>
-      </c>
-      <c r="S43" t="n">
-        <v>0</v>
-      </c>
       <c r="T43" t="n">
         <v>0</v>
       </c>
@@ -3600,10 +3600,10 @@
         <v>0</v>
       </c>
       <c r="V43" t="n">
-        <v>0.0497</v>
+        <v>1.2529</v>
       </c>
       <c r="W43" t="n">
-        <v>1.2529</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -3625,58 +3625,58 @@
         <v>0</v>
       </c>
       <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" t="n">
         <v>0.1264</v>
       </c>
-      <c r="G44" t="n">
-        <v>0</v>
-      </c>
-      <c r="H44" t="n">
-        <v>0</v>
-      </c>
-      <c r="I44" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" t="n">
+      <c r="N44" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="n">
         <v>0.0281</v>
       </c>
-      <c r="K44" t="n">
-        <v>0</v>
-      </c>
-      <c r="L44" t="n">
-        <v>0</v>
-      </c>
-      <c r="M44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N44" t="n">
-        <v>0</v>
-      </c>
-      <c r="O44" t="n">
-        <v>0</v>
-      </c>
-      <c r="P44" t="n">
-        <v>0</v>
-      </c>
       <c r="Q44" t="n">
         <v>0</v>
       </c>
       <c r="R44" t="n">
+        <v>0</v>
+      </c>
+      <c r="S44" t="n">
+        <v>0</v>
+      </c>
+      <c r="T44" t="n">
+        <v>0</v>
+      </c>
+      <c r="U44" t="n">
+        <v>0</v>
+      </c>
+      <c r="V44" t="n">
         <v>0.014</v>
       </c>
-      <c r="S44" t="n">
-        <v>0</v>
-      </c>
-      <c r="T44" t="n">
-        <v>0</v>
-      </c>
-      <c r="U44" t="n">
-        <v>0</v>
-      </c>
-      <c r="V44" t="n">
-        <v>0</v>
-      </c>
       <c r="W44" t="n">
-        <v>0.014</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -3698,46 +3698,46 @@
         <v>0</v>
       </c>
       <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" t="n">
         <v>5.7</v>
       </c>
-      <c r="G45" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" t="n">
-        <v>0</v>
-      </c>
-      <c r="I45" t="n">
-        <v>0</v>
-      </c>
-      <c r="J45" t="n">
-        <v>0</v>
-      </c>
-      <c r="K45" t="n">
+      <c r="N45" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" t="n">
+        <v>0</v>
+      </c>
+      <c r="S45" t="n">
         <v>1.66</v>
-      </c>
-      <c r="L45" t="n">
-        <v>0</v>
-      </c>
-      <c r="M45" t="n">
-        <v>0</v>
-      </c>
-      <c r="N45" t="n">
-        <v>0</v>
-      </c>
-      <c r="O45" t="n">
-        <v>0</v>
-      </c>
-      <c r="P45" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q45" t="n">
-        <v>0</v>
-      </c>
-      <c r="R45" t="n">
-        <v>0</v>
-      </c>
-      <c r="S45" t="n">
-        <v>0</v>
       </c>
       <c r="T45" t="n">
         <v>0</v>
@@ -3765,64 +3765,64 @@
         <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>3.7401</v>
+        <v>1.0731</v>
       </c>
       <c r="E46" t="n">
         <v>0.0018</v>
       </c>
       <c r="F46" t="n">
-        <v>0</v>
+        <v>0.5062</v>
       </c>
       <c r="G46" t="n">
-        <v>0.5062</v>
+        <v>0</v>
       </c>
       <c r="H46" t="n">
+        <v>0.2043</v>
+      </c>
+      <c r="I46" t="n">
+        <v>3.7401</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>9.5472</v>
+      </c>
+      <c r="L46" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0.335</v>
+      </c>
+      <c r="P46" t="n">
+        <v>0.8375</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>0.0074</v>
+      </c>
+      <c r="R46" t="n">
+        <v>0</v>
+      </c>
+      <c r="S46" t="n">
+        <v>0</v>
+      </c>
+      <c r="T46" t="n">
         <v>0.9147999999999999</v>
       </c>
-      <c r="I46" t="n">
-        <v>0.2043</v>
-      </c>
-      <c r="J46" t="n">
-        <v>0.8375</v>
-      </c>
-      <c r="K46" t="n">
-        <v>0</v>
-      </c>
-      <c r="L46" t="n">
-        <v>0</v>
-      </c>
-      <c r="M46" t="n">
-        <v>0</v>
-      </c>
-      <c r="N46" t="n">
-        <v>0</v>
-      </c>
-      <c r="O46" t="n">
+      <c r="U46" t="n">
         <v>0.4638</v>
       </c>
-      <c r="P46" t="n">
-        <v>0.0074</v>
-      </c>
-      <c r="Q46" t="n">
-        <v>1.0731</v>
-      </c>
-      <c r="R46" t="n">
-        <v>0</v>
-      </c>
-      <c r="S46" t="n">
+      <c r="V46" t="n">
+        <v>0</v>
+      </c>
+      <c r="W46" t="n">
         <v>0.0037</v>
-      </c>
-      <c r="T46" t="n">
-        <v>0.335</v>
-      </c>
-      <c r="U46" t="n">
-        <v>9.5472</v>
-      </c>
-      <c r="V46" t="n">
-        <v>0</v>
-      </c>
-      <c r="W46" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -3917,10 +3917,10 @@
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>0</v>
+        <v>0.2437</v>
       </c>
       <c r="G48" t="n">
-        <v>0.2437</v>
+        <v>0</v>
       </c>
       <c r="H48" t="n">
         <v>0</v>
@@ -3929,25 +3929,25 @@
         <v>0</v>
       </c>
       <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" t="n">
         <v>0.0109</v>
-      </c>
-      <c r="K48" t="n">
-        <v>0</v>
-      </c>
-      <c r="L48" t="n">
-        <v>0</v>
-      </c>
-      <c r="M48" t="n">
-        <v>0</v>
-      </c>
-      <c r="N48" t="n">
-        <v>0</v>
-      </c>
-      <c r="O48" t="n">
-        <v>0</v>
-      </c>
-      <c r="P48" t="n">
-        <v>0</v>
       </c>
       <c r="Q48" t="n">
         <v>0</v>
@@ -3996,10 +3996,10 @@
         <v>0</v>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>0.0008</v>
       </c>
       <c r="I49" t="n">
-        <v>0.0008</v>
+        <v>0</v>
       </c>
       <c r="J49" t="n">
         <v>0</v>
@@ -4136,38 +4136,38 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>0</v>
+        <v>0.0019</v>
       </c>
       <c r="G51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" t="n">
         <v>0.0019</v>
       </c>
-      <c r="H51" t="n">
-        <v>0</v>
-      </c>
       <c r="I51" t="n">
-        <v>0.0019</v>
+        <v>0</v>
       </c>
       <c r="J51" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" t="n">
+        <v>0</v>
+      </c>
+      <c r="O51" t="n">
+        <v>0</v>
+      </c>
+      <c r="P51" t="n">
         <v>2.6374</v>
       </c>
-      <c r="K51" t="n">
-        <v>0</v>
-      </c>
-      <c r="L51" t="n">
-        <v>0</v>
-      </c>
-      <c r="M51" t="n">
-        <v>0</v>
-      </c>
-      <c r="N51" t="n">
-        <v>0</v>
-      </c>
-      <c r="O51" t="n">
-        <v>0</v>
-      </c>
-      <c r="P51" t="n">
-        <v>0</v>
-      </c>
       <c r="Q51" t="n">
         <v>0</v>
       </c>
@@ -4184,10 +4184,10 @@
         <v>0</v>
       </c>
       <c r="V51" t="n">
-        <v>0</v>
+        <v>0.0057</v>
       </c>
       <c r="W51" t="n">
-        <v>0.0057</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -4257,10 +4257,10 @@
         <v>0</v>
       </c>
       <c r="V52" t="n">
-        <v>0</v>
+        <v>0.0035</v>
       </c>
       <c r="W52" t="n">
-        <v>0.0035</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -4297,32 +4297,32 @@
         <v>0</v>
       </c>
       <c r="K53" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" t="n">
+        <v>0</v>
+      </c>
+      <c r="M53" t="n">
+        <v>0</v>
+      </c>
+      <c r="N53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" t="n">
+        <v>0</v>
+      </c>
+      <c r="P53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>0</v>
+      </c>
+      <c r="R53" t="n">
+        <v>0</v>
+      </c>
+      <c r="S53" t="n">
         <v>0.3405</v>
       </c>
-      <c r="L53" t="n">
-        <v>0</v>
-      </c>
-      <c r="M53" t="n">
-        <v>0</v>
-      </c>
-      <c r="N53" t="n">
-        <v>0</v>
-      </c>
-      <c r="O53" t="n">
-        <v>0</v>
-      </c>
-      <c r="P53" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q53" t="n">
-        <v>0</v>
-      </c>
-      <c r="R53" t="n">
-        <v>0</v>
-      </c>
-      <c r="S53" t="n">
-        <v>0</v>
-      </c>
       <c r="T53" t="n">
         <v>0</v>
       </c>
@@ -4330,10 +4330,10 @@
         <v>0</v>
       </c>
       <c r="V53" t="n">
-        <v>0</v>
+        <v>0.0185</v>
       </c>
       <c r="W53" t="n">
-        <v>0.0185</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -4349,58 +4349,58 @@
         <v>1</v>
       </c>
       <c r="D54" t="n">
-        <v>0.0154</v>
+        <v>0</v>
       </c>
       <c r="E54" t="n">
         <v>0.0154</v>
       </c>
       <c r="F54" t="n">
-        <v>0</v>
+        <v>0.3547</v>
       </c>
       <c r="G54" t="n">
-        <v>0.3547</v>
+        <v>0.0154</v>
       </c>
       <c r="H54" t="n">
         <v>0</v>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
+        <v>0.0154</v>
       </c>
       <c r="J54" t="n">
         <v>0</v>
       </c>
       <c r="K54" t="n">
-        <v>0</v>
+        <v>0.0308</v>
       </c>
       <c r="L54" t="n">
         <v>0</v>
       </c>
       <c r="M54" t="n">
-        <v>0.0154</v>
+        <v>0</v>
       </c>
       <c r="N54" t="n">
         <v>0</v>
       </c>
       <c r="O54" t="n">
+        <v>1.2645</v>
+      </c>
+      <c r="P54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>0</v>
+      </c>
+      <c r="R54" t="n">
+        <v>0</v>
+      </c>
+      <c r="S54" t="n">
+        <v>0</v>
+      </c>
+      <c r="T54" t="n">
+        <v>0</v>
+      </c>
+      <c r="U54" t="n">
         <v>0.0463</v>
-      </c>
-      <c r="P54" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q54" t="n">
-        <v>0</v>
-      </c>
-      <c r="R54" t="n">
-        <v>0</v>
-      </c>
-      <c r="S54" t="n">
-        <v>0</v>
-      </c>
-      <c r="T54" t="n">
-        <v>1.2645</v>
-      </c>
-      <c r="U54" t="n">
-        <v>0.0308</v>
       </c>
       <c r="V54" t="n">
         <v>0</v>
@@ -4428,58 +4428,58 @@
         <v>2.7089</v>
       </c>
       <c r="F55" t="n">
-        <v>0</v>
+        <v>0.07679999999999999</v>
       </c>
       <c r="G55" t="n">
-        <v>0.07679999999999999</v>
+        <v>8.9337</v>
       </c>
       <c r="H55" t="n">
-        <v>0</v>
+        <v>1.3256</v>
       </c>
       <c r="I55" t="n">
-        <v>1.3256</v>
+        <v>0</v>
       </c>
       <c r="J55" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0.1537</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" t="n">
+        <v>1.3641</v>
+      </c>
+      <c r="P55" t="n">
         <v>0.1921</v>
       </c>
-      <c r="K55" t="n">
-        <v>0</v>
-      </c>
-      <c r="L55" t="n">
-        <v>0</v>
-      </c>
-      <c r="M55" t="n">
-        <v>8.9337</v>
-      </c>
-      <c r="N55" t="n">
+      <c r="Q55" t="n">
+        <v>0.1537</v>
+      </c>
+      <c r="R55" t="n">
         <v>3.1508</v>
       </c>
-      <c r="O55" t="n">
+      <c r="S55" t="n">
+        <v>0</v>
+      </c>
+      <c r="T55" t="n">
+        <v>0</v>
+      </c>
+      <c r="U55" t="n">
         <v>0.1153</v>
       </c>
-      <c r="P55" t="n">
-        <v>0.1537</v>
-      </c>
-      <c r="Q55" t="n">
-        <v>0</v>
-      </c>
-      <c r="R55" t="n">
-        <v>0</v>
-      </c>
-      <c r="S55" t="n">
+      <c r="V55" t="n">
+        <v>0</v>
+      </c>
+      <c r="W55" t="n">
         <v>0.0384</v>
-      </c>
-      <c r="T55" t="n">
-        <v>1.3641</v>
-      </c>
-      <c r="U55" t="n">
-        <v>0.1537</v>
-      </c>
-      <c r="V55" t="n">
-        <v>0</v>
-      </c>
-      <c r="W55" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -4495,64 +4495,64 @@
         <v>1</v>
       </c>
       <c r="D56" t="n">
-        <v>0.007</v>
+        <v>0.0526</v>
       </c>
       <c r="E56" t="n">
         <v>3.0515</v>
       </c>
       <c r="F56" t="n">
-        <v>0</v>
+        <v>0.049</v>
       </c>
       <c r="G56" t="n">
-        <v>0.049</v>
+        <v>10.5735</v>
       </c>
       <c r="H56" t="n">
+        <v>0.9459</v>
+      </c>
+      <c r="I56" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0.0911</v>
+      </c>
+      <c r="L56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" t="n">
+        <v>1.2613</v>
+      </c>
+      <c r="P56" t="n">
+        <v>0.1717</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>0.1331</v>
+      </c>
+      <c r="R56" t="n">
+        <v>3.6191</v>
+      </c>
+      <c r="S56" t="n">
+        <v>0</v>
+      </c>
+      <c r="T56" t="n">
         <v>0.035</v>
       </c>
-      <c r="I56" t="n">
-        <v>0.9459</v>
-      </c>
-      <c r="J56" t="n">
-        <v>0.1717</v>
-      </c>
-      <c r="K56" t="n">
-        <v>0</v>
-      </c>
-      <c r="L56" t="n">
-        <v>0</v>
-      </c>
-      <c r="M56" t="n">
-        <v>10.5735</v>
-      </c>
-      <c r="N56" t="n">
-        <v>3.6191</v>
-      </c>
-      <c r="O56" t="n">
+      <c r="U56" t="n">
         <v>0.0385</v>
       </c>
-      <c r="P56" t="n">
-        <v>0.1331</v>
-      </c>
-      <c r="Q56" t="n">
-        <v>0.0526</v>
-      </c>
-      <c r="R56" t="n">
-        <v>0</v>
-      </c>
-      <c r="S56" t="n">
+      <c r="V56" t="n">
+        <v>0</v>
+      </c>
+      <c r="W56" t="n">
         <v>0.1086</v>
-      </c>
-      <c r="T56" t="n">
-        <v>1.2613</v>
-      </c>
-      <c r="U56" t="n">
-        <v>0.0911</v>
-      </c>
-      <c r="V56" t="n">
-        <v>0</v>
-      </c>
-      <c r="W56" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -4586,25 +4586,25 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" t="n">
+        <v>0</v>
+      </c>
+      <c r="M57" t="n">
+        <v>0</v>
+      </c>
+      <c r="N57" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" t="n">
+        <v>0</v>
+      </c>
+      <c r="P57" t="n">
         <v>0.98</v>
-      </c>
-      <c r="K57" t="n">
-        <v>0</v>
-      </c>
-      <c r="L57" t="n">
-        <v>0</v>
-      </c>
-      <c r="M57" t="n">
-        <v>0</v>
-      </c>
-      <c r="N57" t="n">
-        <v>0</v>
-      </c>
-      <c r="O57" t="n">
-        <v>0</v>
-      </c>
-      <c r="P57" t="n">
-        <v>0</v>
       </c>
       <c r="Q57" t="n">
         <v>0</v>
@@ -4641,58 +4641,58 @@
         <v>1</v>
       </c>
       <c r="D58" t="n">
-        <v>0.0053</v>
+        <v>0</v>
       </c>
       <c r="E58" t="n">
         <v>0.0338</v>
       </c>
       <c r="F58" t="n">
-        <v>0</v>
+        <v>4.7884</v>
       </c>
       <c r="G58" t="n">
-        <v>4.7884</v>
+        <v>0</v>
       </c>
       <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0.0053</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0.0391</v>
+      </c>
+      <c r="L58" t="n">
+        <v>0</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" t="n">
+        <v>0.0587</v>
+      </c>
+      <c r="P58" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q58" t="n">
         <v>0.0036</v>
       </c>
-      <c r="I58" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" t="n">
-        <v>0</v>
-      </c>
-      <c r="K58" t="n">
-        <v>0</v>
-      </c>
-      <c r="L58" t="n">
-        <v>0</v>
-      </c>
-      <c r="M58" t="n">
-        <v>0</v>
-      </c>
-      <c r="N58" t="n">
+      <c r="R58" t="n">
         <v>0.0053</v>
       </c>
-      <c r="O58" t="n">
+      <c r="S58" t="n">
+        <v>0</v>
+      </c>
+      <c r="T58" t="n">
+        <v>0.0036</v>
+      </c>
+      <c r="U58" t="n">
         <v>0.1174</v>
-      </c>
-      <c r="P58" t="n">
-        <v>0.0036</v>
-      </c>
-      <c r="Q58" t="n">
-        <v>0</v>
-      </c>
-      <c r="R58" t="n">
-        <v>0</v>
-      </c>
-      <c r="S58" t="n">
-        <v>0</v>
-      </c>
-      <c r="T58" t="n">
-        <v>0.0587</v>
-      </c>
-      <c r="U58" t="n">
-        <v>0.0391</v>
       </c>
       <c r="V58" t="n">
         <v>0</v>
@@ -4726,37 +4726,37 @@
         <v>0</v>
       </c>
       <c r="H59" t="n">
-        <v>0</v>
+        <v>0.2975</v>
       </c>
       <c r="I59" t="n">
-        <v>0.2975</v>
+        <v>0</v>
       </c>
       <c r="J59" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" t="n">
+        <v>0</v>
+      </c>
+      <c r="M59" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" t="n">
+        <v>0.502</v>
+      </c>
+      <c r="O59" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" t="n">
         <v>0.1488</v>
       </c>
-      <c r="K59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L59" t="n">
-        <v>0</v>
-      </c>
-      <c r="M59" t="n">
-        <v>0</v>
-      </c>
-      <c r="N59" t="n">
-        <v>0</v>
-      </c>
-      <c r="O59" t="n">
-        <v>0</v>
-      </c>
-      <c r="P59" t="n">
-        <v>0</v>
-      </c>
       <c r="Q59" t="n">
         <v>0</v>
       </c>
       <c r="R59" t="n">
-        <v>0.502</v>
+        <v>0</v>
       </c>
       <c r="S59" t="n">
         <v>0</v>
@@ -4793,43 +4793,43 @@
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>0</v>
+        <v>0.0131</v>
       </c>
       <c r="G60" t="n">
-        <v>0.0131</v>
+        <v>0</v>
       </c>
       <c r="H60" t="n">
-        <v>0</v>
+        <v>1.1426</v>
       </c>
       <c r="I60" t="n">
-        <v>1.1426</v>
+        <v>0</v>
       </c>
       <c r="J60" t="n">
+        <v>0</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" t="n">
+        <v>0</v>
+      </c>
+      <c r="M60" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" t="n">
+        <v>0.0218</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0</v>
+      </c>
+      <c r="P60" t="n">
         <v>0.9507</v>
       </c>
-      <c r="K60" t="n">
-        <v>0</v>
-      </c>
-      <c r="L60" t="n">
-        <v>0</v>
-      </c>
-      <c r="M60" t="n">
-        <v>0</v>
-      </c>
-      <c r="N60" t="n">
-        <v>0</v>
-      </c>
-      <c r="O60" t="n">
-        <v>0</v>
-      </c>
-      <c r="P60" t="n">
-        <v>0</v>
-      </c>
       <c r="Q60" t="n">
         <v>0</v>
       </c>
       <c r="R60" t="n">
-        <v>0.0218</v>
+        <v>0</v>
       </c>
       <c r="S60" t="n">
         <v>0</v>
@@ -4841,10 +4841,10 @@
         <v>0</v>
       </c>
       <c r="V60" t="n">
-        <v>0</v>
+        <v>0.0044</v>
       </c>
       <c r="W60" t="n">
-        <v>0.0044</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -4872,31 +4872,31 @@
         <v>0</v>
       </c>
       <c r="H61" t="n">
-        <v>0</v>
+        <v>1.1096</v>
       </c>
       <c r="I61" t="n">
-        <v>1.1096</v>
+        <v>0</v>
       </c>
       <c r="J61" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" t="n">
+        <v>0</v>
+      </c>
+      <c r="M61" t="n">
+        <v>0</v>
+      </c>
+      <c r="N61" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" t="n">
         <v>0.6935</v>
-      </c>
-      <c r="K61" t="n">
-        <v>0</v>
-      </c>
-      <c r="L61" t="n">
-        <v>0</v>
-      </c>
-      <c r="M61" t="n">
-        <v>0</v>
-      </c>
-      <c r="N61" t="n">
-        <v>0</v>
-      </c>
-      <c r="O61" t="n">
-        <v>0</v>
-      </c>
-      <c r="P61" t="n">
-        <v>0</v>
       </c>
       <c r="Q61" t="n">
         <v>0</v>
@@ -4945,31 +4945,31 @@
         <v>0</v>
       </c>
       <c r="H62" t="n">
-        <v>0</v>
+        <v>7.76</v>
       </c>
       <c r="I62" t="n">
-        <v>7.76</v>
+        <v>0</v>
       </c>
       <c r="J62" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" t="n">
+        <v>0</v>
+      </c>
+      <c r="M62" t="n">
+        <v>0</v>
+      </c>
+      <c r="N62" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0</v>
+      </c>
+      <c r="P62" t="n">
         <v>2.2</v>
-      </c>
-      <c r="K62" t="n">
-        <v>0</v>
-      </c>
-      <c r="L62" t="n">
-        <v>0</v>
-      </c>
-      <c r="M62" t="n">
-        <v>0</v>
-      </c>
-      <c r="N62" t="n">
-        <v>0</v>
-      </c>
-      <c r="O62" t="n">
-        <v>0</v>
-      </c>
-      <c r="P62" t="n">
-        <v>0</v>
       </c>
       <c r="Q62" t="n">
         <v>0</v>
@@ -5012,29 +5012,29 @@
         <v>0</v>
       </c>
       <c r="F63" t="n">
+        <v>0.4355</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0</v>
+      </c>
+      <c r="L63" t="n">
+        <v>0</v>
+      </c>
+      <c r="M63" t="n">
         <v>0.5444</v>
       </c>
-      <c r="G63" t="n">
-        <v>0.4355</v>
-      </c>
-      <c r="H63" t="n">
-        <v>0</v>
-      </c>
-      <c r="I63" t="n">
-        <v>0</v>
-      </c>
-      <c r="J63" t="n">
-        <v>0</v>
-      </c>
-      <c r="K63" t="n">
-        <v>0</v>
-      </c>
-      <c r="L63" t="n">
-        <v>0</v>
-      </c>
-      <c r="M63" t="n">
-        <v>0</v>
-      </c>
       <c r="N63" t="n">
         <v>0</v>
       </c>
@@ -5060,10 +5060,10 @@
         <v>0</v>
       </c>
       <c r="V63" t="n">
-        <v>0</v>
+        <v>0.2722</v>
       </c>
       <c r="W63" t="n">
-        <v>0.2722</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -5091,31 +5091,31 @@
         <v>0</v>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>2.18</v>
       </c>
       <c r="I64" t="n">
-        <v>2.18</v>
+        <v>0</v>
       </c>
       <c r="J64" t="n">
+        <v>0</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0</v>
+      </c>
+      <c r="L64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M64" t="n">
+        <v>0</v>
+      </c>
+      <c r="N64" t="n">
+        <v>0</v>
+      </c>
+      <c r="O64" t="n">
+        <v>0</v>
+      </c>
+      <c r="P64" t="n">
         <v>2.63</v>
-      </c>
-      <c r="K64" t="n">
-        <v>0</v>
-      </c>
-      <c r="L64" t="n">
-        <v>0</v>
-      </c>
-      <c r="M64" t="n">
-        <v>0</v>
-      </c>
-      <c r="N64" t="n">
-        <v>0</v>
-      </c>
-      <c r="O64" t="n">
-        <v>0</v>
-      </c>
-      <c r="P64" t="n">
-        <v>0</v>
       </c>
       <c r="Q64" t="n">
         <v>0</v>
@@ -5255,7 +5255,7 @@
         <v>0</v>
       </c>
       <c r="N66" t="n">
-        <v>0</v>
+        <v>0.0688</v>
       </c>
       <c r="O66" t="n">
         <v>0</v>
@@ -5267,7 +5267,7 @@
         <v>0</v>
       </c>
       <c r="R66" t="n">
-        <v>0.0688</v>
+        <v>0</v>
       </c>
       <c r="S66" t="n">
         <v>0</v>
@@ -5310,10 +5310,10 @@
         <v>0</v>
       </c>
       <c r="H67" t="n">
-        <v>0</v>
+        <v>5.23</v>
       </c>
       <c r="I67" t="n">
-        <v>5.23</v>
+        <v>0</v>
       </c>
       <c r="J67" t="n">
         <v>0</v>
@@ -5331,7 +5331,7 @@
         <v>0</v>
       </c>
       <c r="O67" t="n">
-        <v>0</v>
+        <v>5.11</v>
       </c>
       <c r="P67" t="n">
         <v>0</v>
@@ -5346,7 +5346,7 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>5.11</v>
+        <v>0</v>
       </c>
       <c r="U67" t="n">
         <v>0</v>
@@ -5377,37 +5377,37 @@
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>0</v>
+        <v>0.3686</v>
       </c>
       <c r="G68" t="n">
-        <v>0.3686</v>
+        <v>0</v>
       </c>
       <c r="H68" t="n">
-        <v>0</v>
+        <v>0.2183</v>
       </c>
       <c r="I68" t="n">
-        <v>0.2183</v>
+        <v>0</v>
       </c>
       <c r="J68" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" t="n">
+        <v>0</v>
+      </c>
+      <c r="M68" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" t="n">
+        <v>0</v>
+      </c>
+      <c r="O68" t="n">
+        <v>0</v>
+      </c>
+      <c r="P68" t="n">
         <v>3.0508</v>
-      </c>
-      <c r="K68" t="n">
-        <v>0</v>
-      </c>
-      <c r="L68" t="n">
-        <v>0</v>
-      </c>
-      <c r="M68" t="n">
-        <v>0</v>
-      </c>
-      <c r="N68" t="n">
-        <v>0</v>
-      </c>
-      <c r="O68" t="n">
-        <v>0</v>
-      </c>
-      <c r="P68" t="n">
-        <v>0</v>
       </c>
       <c r="Q68" t="n">
         <v>0</v>
@@ -5477,7 +5477,7 @@
         <v>0</v>
       </c>
       <c r="O69" t="n">
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="P69" t="n">
         <v>0</v>
@@ -5489,19 +5489,19 @@
         <v>0</v>
       </c>
       <c r="S69" t="n">
+        <v>0</v>
+      </c>
+      <c r="T69" t="n">
+        <v>0</v>
+      </c>
+      <c r="U69" t="n">
+        <v>0</v>
+      </c>
+      <c r="V69" t="n">
+        <v>0</v>
+      </c>
+      <c r="W69" t="n">
         <v>2.3</v>
-      </c>
-      <c r="T69" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="U69" t="n">
-        <v>0</v>
-      </c>
-      <c r="V69" t="n">
-        <v>0</v>
-      </c>
-      <c r="W69" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -5547,7 +5547,7 @@
         <v>0</v>
       </c>
       <c r="N70" t="n">
-        <v>0</v>
+        <v>0.72</v>
       </c>
       <c r="O70" t="n">
         <v>0</v>
@@ -5559,7 +5559,7 @@
         <v>0</v>
       </c>
       <c r="R70" t="n">
-        <v>0.72</v>
+        <v>0</v>
       </c>
       <c r="S70" t="n">
         <v>0</v>
@@ -5611,31 +5611,31 @@
         <v>0</v>
       </c>
       <c r="K71" t="n">
+        <v>0</v>
+      </c>
+      <c r="L71" t="n">
+        <v>0</v>
+      </c>
+      <c r="M71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" t="n">
+        <v>0.0506</v>
+      </c>
+      <c r="O71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>0</v>
+      </c>
+      <c r="R71" t="n">
+        <v>0</v>
+      </c>
+      <c r="S71" t="n">
         <v>0.1935</v>
-      </c>
-      <c r="L71" t="n">
-        <v>0</v>
-      </c>
-      <c r="M71" t="n">
-        <v>0</v>
-      </c>
-      <c r="N71" t="n">
-        <v>0</v>
-      </c>
-      <c r="O71" t="n">
-        <v>0</v>
-      </c>
-      <c r="P71" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q71" t="n">
-        <v>0</v>
-      </c>
-      <c r="R71" t="n">
-        <v>0.0506</v>
-      </c>
-      <c r="S71" t="n">
-        <v>0</v>
       </c>
       <c r="T71" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
updating files for mantenance
</commit_message>
<xml_diff>
--- a/data/Influencers_OLS.xlsx
+++ b/data/Influencers_OLS.xlsx
@@ -441,102 +441,102 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>214</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>23</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>526</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>565</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>625</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>678</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>863</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>871</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>351</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>334</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>725</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>471</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>375</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>584</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>408</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>871</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>549</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>864</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>712</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>214</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>351</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>229</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>863</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>565</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>625</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>526</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>471</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>375</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>725</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>678</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>0.1508</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -595,7 +595,7 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>0.1508</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
         <v>0</v>
@@ -635,52 +635,52 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="n">
         <v>2.48</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U3" t="n">
-        <v>2.42</v>
-      </c>
-      <c r="V3" t="n">
-        <v>0</v>
       </c>
       <c r="W3" t="n">
         <v>0</v>
@@ -699,7 +699,7 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>0.921</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -708,52 +708,52 @@
         <v>0.0767</v>
       </c>
       <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>11.9724</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>5.8839</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.0767</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="n">
         <v>0.2047</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.921</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="n">
-        <v>11.9724</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0.0767</v>
-      </c>
-      <c r="S4" t="n">
-        <v>5.8839</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V4" t="n">
-        <v>0</v>
       </c>
       <c r="W4" t="n">
         <v>0</v>
@@ -772,61 +772,61 @@
         <v>3</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>0.3021</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
+        <v>0.0336</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.1394</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1.1592</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="n">
         <v>0.1188</v>
       </c>
-      <c r="G5" t="n">
+      <c r="U5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" t="n">
         <v>0.07489999999999999</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.3021</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.1394</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" t="n">
-        <v>0.0336</v>
-      </c>
-      <c r="S5" t="n">
-        <v>1.1592</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" t="n">
-        <v>0</v>
       </c>
       <c r="W5" t="n">
         <v>0</v>
@@ -845,61 +845,61 @@
         <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>0.6947</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.8535</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.5558</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
         <v>0.0595</v>
       </c>
-      <c r="G6" t="n">
+      <c r="U6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" t="n">
         <v>3.156</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.6947</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.8535</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.5558</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0</v>
       </c>
       <c r="W6" t="n">
         <v>0</v>
@@ -918,61 +918,61 @@
         <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>13.5058</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
+        <v>1.2431</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.9051</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.1512</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
         <v>0.0504</v>
       </c>
-      <c r="G7" t="n">
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" t="n">
         <v>0.168</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
-        <v>13.5058</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="n">
-        <v>4.9051</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" t="n">
-        <v>1.2431</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0.1512</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" t="n">
-        <v>0</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
@@ -991,61 +991,61 @@
         <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>3.6515</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
+        <v>1.2749</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2.7326</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.3656</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
         <v>2.3622</v>
       </c>
-      <c r="G8" t="n">
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" t="n">
         <v>0.3127</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
-        <v>3.6515</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="n">
-        <v>2.7326</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" t="n">
-        <v>1.2749</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0.3656</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" t="n">
-        <v>0</v>
-      </c>
-      <c r="V8" t="n">
-        <v>0</v>
       </c>
       <c r="W8" t="n">
         <v>0</v>
@@ -1064,61 +1064,61 @@
         <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
+        <v>0.1686</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.9258999999999999</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.2541</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" t="n">
         <v>0.08550000000000001</v>
       </c>
-      <c r="G9" t="n">
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" t="n">
         <v>3.4666</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.9429999999999999</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0.9258999999999999</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0.1686</v>
-      </c>
-      <c r="S9" t="n">
-        <v>0.2541</v>
-      </c>
-      <c r="T9" t="n">
-        <v>0</v>
-      </c>
-      <c r="U9" t="n">
-        <v>0</v>
-      </c>
-      <c r="V9" t="n">
-        <v>0</v>
       </c>
       <c r="W9" t="n">
         <v>0</v>
@@ -1155,40 +1155,40 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" t="n">
         <v>0.1059</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U10" t="n">
-        <v>0</v>
       </c>
       <c r="V10" t="n">
         <v>0</v>
@@ -1210,28 +1210,28 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
         <v>0.151</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.2643</v>
+      </c>
+      <c r="H11" t="n">
         <v>0.0126</v>
       </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
       <c r="I11" t="n">
-        <v>2.7054</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2517</v>
+        <v>0.0126</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>1.661</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -1240,34 +1240,34 @@
         <v>0.4404</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>0.0126</v>
       </c>
       <c r="O11" t="n">
-        <v>1.661</v>
+        <v>0.1762</v>
       </c>
       <c r="P11" t="n">
-        <v>0.2643</v>
+        <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.0126</v>
+        <v>1.8498</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>0</v>
+        <v>0.7927999999999999</v>
       </c>
       <c r="T11" t="n">
-        <v>0.7927999999999999</v>
+        <v>0</v>
       </c>
       <c r="U11" t="n">
-        <v>1.8498</v>
+        <v>0.2517</v>
       </c>
       <c r="V11" t="n">
-        <v>0.1762</v>
+        <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>0.0126</v>
+        <v>2.7054</v>
       </c>
     </row>
     <row r="12">
@@ -1298,7 +1298,7 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>0.0029</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -1313,7 +1313,7 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>0.0029</v>
+        <v>0</v>
       </c>
       <c r="O12" t="n">
         <v>0</v>
@@ -1356,28 +1356,28 @@
         <v>1</v>
       </c>
       <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
         <v>1.2332</v>
       </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>0.2466</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>0.3035</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>3.2821</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>2.1628</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -1389,31 +1389,31 @@
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>2.1628</v>
+        <v>0.3035</v>
       </c>
       <c r="P13" t="n">
-        <v>0.2466</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>0.1138</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>0</v>
+        <v>0.702</v>
       </c>
       <c r="T13" t="n">
-        <v>0.702</v>
+        <v>0</v>
       </c>
       <c r="U13" t="n">
-        <v>0.1138</v>
+        <v>3.2821</v>
       </c>
       <c r="V13" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" t="n">
         <v>0.3035</v>
-      </c>
-      <c r="W13" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1468,7 +1468,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>0.0144</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
@@ -1480,7 +1480,7 @@
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>0.0144</v>
+        <v>0</v>
       </c>
       <c r="V14" t="n">
         <v>0</v>
@@ -1514,7 +1514,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>0.295</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -1523,7 +1523,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>0.0047</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -1535,13 +1535,13 @@
         <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>0.0047</v>
+        <v>0</v>
       </c>
       <c r="P15" t="n">
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.295</v>
+        <v>0</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
@@ -1575,61 +1575,61 @@
         <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1.3715</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
+        <v>0.0867</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.8999</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0.7877</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" t="n">
         <v>0.1326</v>
       </c>
-      <c r="G16" t="n">
+      <c r="U16" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" t="n">
         <v>0.4334</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="n">
-        <v>1.3715</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0.8999</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" t="n">
-        <v>0.0867</v>
-      </c>
-      <c r="S16" t="n">
-        <v>0.7877</v>
-      </c>
-      <c r="T16" t="n">
-        <v>0</v>
-      </c>
-      <c r="U16" t="n">
-        <v>0</v>
-      </c>
-      <c r="V16" t="n">
-        <v>0</v>
       </c>
       <c r="W16" t="n">
         <v>0</v>
@@ -1648,7 +1648,7 @@
         <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>3.2514</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -1657,52 +1657,52 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>2.605</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" t="n">
         <v>0.3597</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="n">
-        <v>3.2514</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" t="n">
-        <v>2.605</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" t="n">
-        <v>0</v>
-      </c>
-      <c r="T17" t="n">
-        <v>0</v>
-      </c>
-      <c r="U17" t="n">
-        <v>0</v>
-      </c>
-      <c r="V17" t="n">
-        <v>0</v>
       </c>
       <c r="W17" t="n">
         <v>0</v>
@@ -1721,46 +1721,46 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
         <v>0.005</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="n">
         <v>0.009900000000000001</v>
       </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" t="n">
-        <v>0</v>
-      </c>
       <c r="O18" t="n">
-        <v>0.0298</v>
+        <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.005</v>
+        <v>0.0944</v>
       </c>
       <c r="R18" t="n">
         <v>0</v>
@@ -1772,7 +1772,7 @@
         <v>0</v>
       </c>
       <c r="U18" t="n">
-        <v>0.0944</v>
+        <v>0</v>
       </c>
       <c r="V18" t="n">
         <v>0</v>
@@ -1803,19 +1803,19 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0.0259</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>0.0029</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>0.3076</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
@@ -1824,16 +1824,16 @@
         <v>0.06610000000000001</v>
       </c>
       <c r="N19" t="n">
-        <v>0.0029</v>
+        <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>0.3076</v>
+        <v>0</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>0</v>
+        <v>0.8107</v>
       </c>
       <c r="R19" t="n">
         <v>0</v>
@@ -1845,10 +1845,10 @@
         <v>0</v>
       </c>
       <c r="U19" t="n">
-        <v>0.8107</v>
+        <v>0</v>
       </c>
       <c r="V19" t="n">
-        <v>0</v>
+        <v>0.0259</v>
       </c>
       <c r="W19" t="n">
         <v>0</v>
@@ -1879,52 +1879,52 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>0.0013</v>
       </c>
       <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" t="n">
+        <v>0</v>
+      </c>
+      <c r="W20" t="n">
         <v>0.3998</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>0.0013</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" t="n">
-        <v>0</v>
-      </c>
-      <c r="T20" t="n">
-        <v>0</v>
-      </c>
-      <c r="U20" t="n">
-        <v>0</v>
-      </c>
-      <c r="V20" t="n">
-        <v>0</v>
-      </c>
-      <c r="W20" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -2013,64 +2013,64 @@
         <v>1</v>
       </c>
       <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
         <v>0.0391</v>
       </c>
-      <c r="E22" t="n">
-        <v>1.7373</v>
-      </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>0.0117</v>
       </c>
       <c r="H22" t="n">
+        <v>0.4617</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
+        <v>1.4986</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.2191</v>
+      </c>
+      <c r="L22" t="n">
         <v>0.4069</v>
-      </c>
-      <c r="I22" t="n">
-        <v>7.1605</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0.043</v>
-      </c>
-      <c r="K22" t="n">
-        <v>1.4751</v>
-      </c>
-      <c r="L22" t="n">
-        <v>0</v>
       </c>
       <c r="M22" t="n">
         <v>0.0157</v>
       </c>
       <c r="N22" t="n">
-        <v>0</v>
+        <v>1.7373</v>
       </c>
       <c r="O22" t="n">
-        <v>0.2191</v>
+        <v>0.0078</v>
       </c>
       <c r="P22" t="n">
-        <v>0.0117</v>
+        <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.4617</v>
+        <v>5.1571</v>
       </c>
       <c r="R22" t="n">
-        <v>0</v>
+        <v>1.4751</v>
       </c>
       <c r="S22" t="n">
-        <v>0</v>
+        <v>0.1683</v>
       </c>
       <c r="T22" t="n">
-        <v>0.1683</v>
+        <v>0</v>
       </c>
       <c r="U22" t="n">
-        <v>5.1571</v>
+        <v>0.043</v>
       </c>
       <c r="V22" t="n">
-        <v>0.0078</v>
+        <v>0</v>
       </c>
       <c r="W22" t="n">
-        <v>1.4986</v>
+        <v>7.1605</v>
       </c>
     </row>
     <row r="23">
@@ -2086,61 +2086,61 @@
         <v>3</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>0.1151</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
+        <v>0.0192</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.5757</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.1343</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" t="n">
+        <v>0</v>
+      </c>
+      <c r="T23" t="n">
         <v>1.8231</v>
       </c>
-      <c r="G23" t="n">
+      <c r="U23" t="n">
+        <v>0</v>
+      </c>
+      <c r="V23" t="n">
         <v>0.2687</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0.1151</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0.5757</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" t="n">
-        <v>0.0192</v>
-      </c>
-      <c r="S23" t="n">
-        <v>0.1343</v>
-      </c>
-      <c r="T23" t="n">
-        <v>0</v>
-      </c>
-      <c r="U23" t="n">
-        <v>0</v>
-      </c>
-      <c r="V23" t="n">
-        <v>0</v>
       </c>
       <c r="W23" t="n">
         <v>0</v>
@@ -2159,28 +2159,28 @@
         <v>1</v>
       </c>
       <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
         <v>0.3069</v>
       </c>
-      <c r="E24" t="n">
-        <v>0</v>
-      </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>1.4854</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>0.3069</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>0.2946</v>
+        <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>0.0123</v>
+        <v>0.8102</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -2192,31 +2192,31 @@
         <v>0</v>
       </c>
       <c r="O24" t="n">
-        <v>0.8102</v>
+        <v>3.5846</v>
       </c>
       <c r="P24" t="n">
-        <v>1.4854</v>
+        <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>0</v>
+        <v>0.2332</v>
       </c>
       <c r="R24" t="n">
-        <v>0</v>
+        <v>0.0123</v>
       </c>
       <c r="S24" t="n">
-        <v>0</v>
+        <v>0.6875</v>
       </c>
       <c r="T24" t="n">
-        <v>0.6875</v>
+        <v>0</v>
       </c>
       <c r="U24" t="n">
-        <v>0.2332</v>
+        <v>0.2946</v>
       </c>
       <c r="V24" t="n">
-        <v>3.5846</v>
+        <v>0</v>
       </c>
       <c r="W24" t="n">
-        <v>0</v>
+        <v>0.3069</v>
       </c>
     </row>
     <row r="25">
@@ -2232,7 +2232,7 @@
         <v>2</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>0.1928</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -2241,13 +2241,13 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>0.1704</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>0.1748</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -2256,13 +2256,13 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>0.1928</v>
+        <v>0</v>
       </c>
       <c r="M25" t="n">
         <v>0.7262999999999999</v>
       </c>
       <c r="N25" t="n">
-        <v>0.1748</v>
+        <v>0</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
@@ -2286,7 +2286,7 @@
         <v>0</v>
       </c>
       <c r="V25" t="n">
-        <v>0</v>
+        <v>0.1704</v>
       </c>
       <c r="W25" t="n">
         <v>0</v>
@@ -2384,55 +2384,55 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>0.0395</v>
       </c>
       <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.06909999999999999</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="n">
+        <v>0</v>
+      </c>
+      <c r="T27" t="n">
+        <v>0</v>
+      </c>
+      <c r="U27" t="n">
+        <v>0</v>
+      </c>
+      <c r="V27" t="n">
         <v>0.0395</v>
-      </c>
-      <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" t="n">
-        <v>0.06909999999999999</v>
-      </c>
-      <c r="O27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" t="n">
-        <v>0.0395</v>
-      </c>
-      <c r="S27" t="n">
-        <v>0</v>
-      </c>
-      <c r="T27" t="n">
-        <v>0</v>
-      </c>
-      <c r="U27" t="n">
-        <v>0</v>
-      </c>
-      <c r="V27" t="n">
-        <v>0</v>
       </c>
       <c r="W27" t="n">
         <v>0</v>
@@ -2460,52 +2460,52 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.948</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0.5959</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" t="n">
         <v>0.0271</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" t="n">
-        <v>0.948</v>
-      </c>
-      <c r="P28" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" t="n">
-        <v>0</v>
-      </c>
-      <c r="S28" t="n">
-        <v>0</v>
-      </c>
-      <c r="T28" t="n">
-        <v>0</v>
-      </c>
-      <c r="U28" t="n">
-        <v>0.5959</v>
-      </c>
-      <c r="V28" t="n">
-        <v>0</v>
       </c>
       <c r="W28" t="n">
         <v>0</v>
@@ -2530,7 +2530,7 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>3.1</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
@@ -2539,7 +2539,7 @@
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>0.55</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -2554,7 +2554,7 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>0.55</v>
+        <v>0</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
@@ -2566,7 +2566,7 @@
         <v>0</v>
       </c>
       <c r="R29" t="n">
-        <v>3.1</v>
+        <v>0</v>
       </c>
       <c r="S29" t="n">
         <v>0</v>
@@ -2606,16 +2606,16 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>0.2099</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>0.0036</v>
       </c>
       <c r="I30" t="n">
-        <v>1.4328</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>3.0972</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -2633,28 +2633,28 @@
         <v>0</v>
       </c>
       <c r="P30" t="n">
-        <v>0.2099</v>
+        <v>0</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.0036</v>
+        <v>0.0145</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>0</v>
+        <v>0.5934</v>
       </c>
       <c r="T30" t="n">
-        <v>0.5934</v>
+        <v>0</v>
       </c>
       <c r="U30" t="n">
-        <v>0.0145</v>
+        <v>0</v>
       </c>
       <c r="V30" t="n">
         <v>0</v>
       </c>
       <c r="W30" t="n">
-        <v>3.0972</v>
+        <v>1.4328</v>
       </c>
     </row>
     <row r="31">
@@ -2679,7 +2679,7 @@
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0511</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -2691,7 +2691,7 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>0.4151</v>
       </c>
       <c r="L31" t="n">
         <v>0</v>
@@ -2703,13 +2703,13 @@
         <v>0</v>
       </c>
       <c r="O31" t="n">
-        <v>0.4151</v>
+        <v>0</v>
       </c>
       <c r="P31" t="n">
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>0</v>
+        <v>0.2917</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2721,10 +2721,10 @@
         <v>0</v>
       </c>
       <c r="U31" t="n">
-        <v>0.2917</v>
+        <v>0</v>
       </c>
       <c r="V31" t="n">
-        <v>0</v>
+        <v>0.0511</v>
       </c>
       <c r="W31" t="n">
         <v>0</v>
@@ -2752,7 +2752,7 @@
         <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>0.0277</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -2764,7 +2764,7 @@
         <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>0</v>
+        <v>0.8921</v>
       </c>
       <c r="L32" t="n">
         <v>0</v>
@@ -2776,13 +2776,13 @@
         <v>0</v>
       </c>
       <c r="O32" t="n">
-        <v>0.8921</v>
+        <v>0</v>
       </c>
       <c r="P32" t="n">
         <v>0</v>
       </c>
       <c r="Q32" t="n">
-        <v>0</v>
+        <v>0.1908</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2794,10 +2794,10 @@
         <v>0</v>
       </c>
       <c r="U32" t="n">
-        <v>0.1908</v>
+        <v>0</v>
       </c>
       <c r="V32" t="n">
-        <v>0</v>
+        <v>0.0277</v>
       </c>
       <c r="W32" t="n">
         <v>0</v>
@@ -2816,7 +2816,7 @@
         <v>2</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>0.5633</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
@@ -2825,31 +2825,31 @@
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0129</v>
+        <v>0</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>0.0493</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>0.0107</v>
       </c>
       <c r="L33" t="n">
-        <v>0.5633</v>
+        <v>0</v>
       </c>
       <c r="M33" t="n">
         <v>0.0278</v>
       </c>
       <c r="N33" t="n">
-        <v>0.0493</v>
+        <v>0</v>
       </c>
       <c r="O33" t="n">
-        <v>0.0107</v>
+        <v>0</v>
       </c>
       <c r="P33" t="n">
         <v>0</v>
@@ -2870,7 +2870,7 @@
         <v>0</v>
       </c>
       <c r="V33" t="n">
-        <v>0</v>
+        <v>0.0129</v>
       </c>
       <c r="W33" t="n">
         <v>0</v>
@@ -2889,7 +2889,7 @@
         <v>2</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>0.0774</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
@@ -2898,31 +2898,31 @@
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>0.1065</v>
+        <v>0</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>0.19</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>0.0182</v>
       </c>
       <c r="L34" t="n">
-        <v>0.0774</v>
+        <v>0</v>
       </c>
       <c r="M34" t="n">
         <v>0.0339</v>
       </c>
       <c r="N34" t="n">
-        <v>0.19</v>
+        <v>0</v>
       </c>
       <c r="O34" t="n">
-        <v>0.0182</v>
+        <v>0</v>
       </c>
       <c r="P34" t="n">
         <v>0</v>
@@ -2943,7 +2943,7 @@
         <v>0</v>
       </c>
       <c r="V34" t="n">
-        <v>0</v>
+        <v>0.1065</v>
       </c>
       <c r="W34" t="n">
         <v>0</v>
@@ -2962,28 +2962,28 @@
         <v>1</v>
       </c>
       <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
         <v>2.2016</v>
       </c>
-      <c r="E35" t="n">
-        <v>0.0022</v>
-      </c>
       <c r="F35" t="n">
         <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>0</v>
+        <v>4.4009</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>0.0044</v>
       </c>
       <c r="I35" t="n">
-        <v>0.2292</v>
+        <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>2.8605</v>
+        <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>1.536</v>
       </c>
       <c r="L35" t="n">
         <v>0</v>
@@ -2992,34 +2992,34 @@
         <v>5.0709</v>
       </c>
       <c r="N35" t="n">
-        <v>0</v>
+        <v>0.0022</v>
       </c>
       <c r="O35" t="n">
-        <v>1.536</v>
+        <v>2.0539</v>
       </c>
       <c r="P35" t="n">
-        <v>4.4009</v>
+        <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>0.0044</v>
+        <v>0.141</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>0</v>
+        <v>0.6016</v>
       </c>
       <c r="T35" t="n">
-        <v>0.6016</v>
+        <v>0</v>
       </c>
       <c r="U35" t="n">
-        <v>0.141</v>
+        <v>2.8605</v>
       </c>
       <c r="V35" t="n">
-        <v>2.0539</v>
+        <v>0</v>
       </c>
       <c r="W35" t="n">
-        <v>0</v>
+        <v>0.2292</v>
       </c>
     </row>
     <row r="36">
@@ -3041,7 +3041,7 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>1.8556</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -3077,7 +3077,7 @@
         <v>0</v>
       </c>
       <c r="R36" t="n">
-        <v>1.8556</v>
+        <v>0</v>
       </c>
       <c r="S36" t="n">
         <v>0</v>
@@ -3129,7 +3129,7 @@
         <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>0.0263</v>
       </c>
       <c r="L37" t="n">
         <v>0</v>
@@ -3141,13 +3141,13 @@
         <v>0</v>
       </c>
       <c r="O37" t="n">
-        <v>0.0263</v>
+        <v>0</v>
       </c>
       <c r="P37" t="n">
         <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>0</v>
+        <v>0.0075</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3159,7 +3159,7 @@
         <v>0</v>
       </c>
       <c r="U37" t="n">
-        <v>0.0075</v>
+        <v>0</v>
       </c>
       <c r="V37" t="n">
         <v>0</v>
@@ -3181,7 +3181,7 @@
         <v>2</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>4.2629</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
@@ -3190,13 +3190,13 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>0.168</v>
+        <v>0</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>1.008</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -3205,13 +3205,13 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>4.2629</v>
+        <v>0</v>
       </c>
       <c r="M38" t="n">
         <v>0.63</v>
       </c>
       <c r="N38" t="n">
-        <v>1.008</v>
+        <v>0</v>
       </c>
       <c r="O38" t="n">
         <v>0</v>
@@ -3235,7 +3235,7 @@
         <v>0</v>
       </c>
       <c r="V38" t="n">
-        <v>0</v>
+        <v>0.168</v>
       </c>
       <c r="W38" t="n">
         <v>0</v>
@@ -3254,7 +3254,7 @@
         <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>0.0493</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
@@ -3263,31 +3263,31 @@
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>0.009900000000000001</v>
+        <v>0</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>0.1675</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>0.0985</v>
       </c>
       <c r="L39" t="n">
-        <v>0.0493</v>
+        <v>0</v>
       </c>
       <c r="M39" t="n">
         <v>0.0197</v>
       </c>
       <c r="N39" t="n">
-        <v>0.1675</v>
+        <v>0</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0985</v>
+        <v>0</v>
       </c>
       <c r="P39" t="n">
         <v>0</v>
@@ -3308,7 +3308,7 @@
         <v>0</v>
       </c>
       <c r="V39" t="n">
-        <v>0</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="W39" t="n">
         <v>0</v>
@@ -3327,7 +3327,7 @@
         <v>3</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>4.41</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
@@ -3351,7 +3351,7 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>4.41</v>
+        <v>0</v>
       </c>
       <c r="M40" t="n">
         <v>0</v>
@@ -3439,7 +3439,7 @@
         <v>0</v>
       </c>
       <c r="Q41" t="n">
-        <v>0</v>
+        <v>0.0013</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3451,7 +3451,7 @@
         <v>0</v>
       </c>
       <c r="U41" t="n">
-        <v>0.0013</v>
+        <v>0</v>
       </c>
       <c r="V41" t="n">
         <v>0</v>
@@ -3494,7 +3494,7 @@
         <v>0</v>
       </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>0.0431</v>
       </c>
       <c r="L42" t="n">
         <v>0</v>
@@ -3506,7 +3506,7 @@
         <v>0</v>
       </c>
       <c r="O42" t="n">
-        <v>0.0431</v>
+        <v>0</v>
       </c>
       <c r="P42" t="n">
         <v>0</v>
@@ -3546,61 +3546,61 @@
         <v>3</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>0.0975</v>
       </c>
       <c r="E43" t="n">
         <v>0</v>
       </c>
       <c r="F43" t="n">
+        <v>0.0139</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="n">
+        <v>1.2529</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" t="n">
+        <v>0.0497</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>0</v>
+      </c>
+      <c r="R43" t="n">
+        <v>0</v>
+      </c>
+      <c r="S43" t="n">
+        <v>0</v>
+      </c>
+      <c r="T43" t="n">
         <v>0.5569</v>
       </c>
-      <c r="G43" t="n">
+      <c r="U43" t="n">
+        <v>0</v>
+      </c>
+      <c r="V43" t="n">
         <v>0.0975</v>
-      </c>
-      <c r="H43" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" t="n">
-        <v>0</v>
-      </c>
-      <c r="K43" t="n">
-        <v>0</v>
-      </c>
-      <c r="L43" t="n">
-        <v>0.0975</v>
-      </c>
-      <c r="M43" t="n">
-        <v>0</v>
-      </c>
-      <c r="N43" t="n">
-        <v>1.2529</v>
-      </c>
-      <c r="O43" t="n">
-        <v>0</v>
-      </c>
-      <c r="P43" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q43" t="n">
-        <v>0</v>
-      </c>
-      <c r="R43" t="n">
-        <v>0.0139</v>
-      </c>
-      <c r="S43" t="n">
-        <v>0.0497</v>
-      </c>
-      <c r="T43" t="n">
-        <v>0</v>
-      </c>
-      <c r="U43" t="n">
-        <v>0</v>
-      </c>
-      <c r="V43" t="n">
-        <v>0</v>
       </c>
       <c r="W43" t="n">
         <v>0</v>
@@ -3619,7 +3619,7 @@
         <v>2</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>0.1264</v>
       </c>
       <c r="E44" t="n">
         <v>0</v>
@@ -3628,52 +3628,52 @@
         <v>0</v>
       </c>
       <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="n">
         <v>0.014</v>
       </c>
-      <c r="H44" t="n">
-        <v>0</v>
-      </c>
-      <c r="I44" t="n">
-        <v>0</v>
-      </c>
       <c r="J44" t="n">
         <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>0.0281</v>
       </c>
       <c r="L44" t="n">
-        <v>0.1264</v>
+        <v>0</v>
       </c>
       <c r="M44" t="n">
         <v>0</v>
       </c>
       <c r="N44" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>0</v>
+      </c>
+      <c r="R44" t="n">
+        <v>0</v>
+      </c>
+      <c r="S44" t="n">
+        <v>0</v>
+      </c>
+      <c r="T44" t="n">
+        <v>0</v>
+      </c>
+      <c r="U44" t="n">
+        <v>0</v>
+      </c>
+      <c r="V44" t="n">
         <v>0.014</v>
-      </c>
-      <c r="O44" t="n">
-        <v>0.0281</v>
-      </c>
-      <c r="P44" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q44" t="n">
-        <v>0</v>
-      </c>
-      <c r="R44" t="n">
-        <v>0</v>
-      </c>
-      <c r="S44" t="n">
-        <v>0</v>
-      </c>
-      <c r="T44" t="n">
-        <v>0</v>
-      </c>
-      <c r="U44" t="n">
-        <v>0</v>
-      </c>
-      <c r="V44" t="n">
-        <v>0</v>
       </c>
       <c r="W44" t="n">
         <v>0</v>
@@ -3692,13 +3692,13 @@
         <v>3</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>5.7</v>
       </c>
       <c r="E45" t="n">
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>0</v>
+        <v>1.66</v>
       </c>
       <c r="G45" t="n">
         <v>0</v>
@@ -3716,7 +3716,7 @@
         <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
       <c r="M45" t="n">
         <v>0</v>
@@ -3734,7 +3734,7 @@
         <v>0</v>
       </c>
       <c r="R45" t="n">
-        <v>1.66</v>
+        <v>0</v>
       </c>
       <c r="S45" t="n">
         <v>0</v>
@@ -3765,64 +3765,64 @@
         <v>1</v>
       </c>
       <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
         <v>0.9147999999999999</v>
       </c>
-      <c r="E46" t="n">
-        <v>0.0037</v>
-      </c>
       <c r="F46" t="n">
         <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>0</v>
+        <v>1.0731</v>
       </c>
       <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0.0074</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0.8375</v>
+      </c>
+      <c r="L46" t="n">
         <v>0.0018</v>
-      </c>
-      <c r="I46" t="n">
-        <v>0.335</v>
-      </c>
-      <c r="J46" t="n">
-        <v>0.4638</v>
-      </c>
-      <c r="K46" t="n">
-        <v>0</v>
-      </c>
-      <c r="L46" t="n">
-        <v>0</v>
       </c>
       <c r="M46" t="n">
         <v>0.5062</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
+        <v>0.0037</v>
       </c>
       <c r="O46" t="n">
-        <v>0.8375</v>
+        <v>3.7401</v>
       </c>
       <c r="P46" t="n">
-        <v>1.0731</v>
+        <v>0</v>
       </c>
       <c r="Q46" t="n">
-        <v>0</v>
+        <v>0.2043</v>
       </c>
       <c r="R46" t="n">
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>0</v>
+        <v>9.5472</v>
       </c>
       <c r="T46" t="n">
-        <v>9.5472</v>
+        <v>0</v>
       </c>
       <c r="U46" t="n">
-        <v>0.2043</v>
+        <v>0.4638</v>
       </c>
       <c r="V46" t="n">
-        <v>3.7401</v>
+        <v>0</v>
       </c>
       <c r="W46" t="n">
-        <v>0.0074</v>
+        <v>0.335</v>
       </c>
     </row>
     <row r="47">
@@ -3932,7 +3932,7 @@
         <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>0</v>
+        <v>0.0109</v>
       </c>
       <c r="L48" t="n">
         <v>0</v>
@@ -3944,7 +3944,7 @@
         <v>0</v>
       </c>
       <c r="O48" t="n">
-        <v>0.0109</v>
+        <v>0</v>
       </c>
       <c r="P48" t="n">
         <v>0</v>
@@ -4023,7 +4023,7 @@
         <v>0</v>
       </c>
       <c r="Q49" t="n">
-        <v>0</v>
+        <v>0.0008</v>
       </c>
       <c r="R49" t="n">
         <v>0</v>
@@ -4035,7 +4035,7 @@
         <v>0</v>
       </c>
       <c r="U49" t="n">
-        <v>0.0008</v>
+        <v>0</v>
       </c>
       <c r="V49" t="n">
         <v>0</v>
@@ -4145,13 +4145,13 @@
         <v>0</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
+        <v>0.0057</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
       </c>
       <c r="K51" t="n">
-        <v>0</v>
+        <v>2.6374</v>
       </c>
       <c r="L51" t="n">
         <v>0</v>
@@ -4160,16 +4160,16 @@
         <v>0.0019</v>
       </c>
       <c r="N51" t="n">
-        <v>0.0057</v>
+        <v>0</v>
       </c>
       <c r="O51" t="n">
-        <v>2.6374</v>
+        <v>0</v>
       </c>
       <c r="P51" t="n">
         <v>0</v>
       </c>
       <c r="Q51" t="n">
-        <v>0</v>
+        <v>0.0019</v>
       </c>
       <c r="R51" t="n">
         <v>0</v>
@@ -4181,7 +4181,7 @@
         <v>0</v>
       </c>
       <c r="U51" t="n">
-        <v>0.0019</v>
+        <v>0</v>
       </c>
       <c r="V51" t="n">
         <v>0</v>
@@ -4218,7 +4218,7 @@
         <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>0</v>
+        <v>0.0035</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -4233,7 +4233,7 @@
         <v>0</v>
       </c>
       <c r="N52" t="n">
-        <v>0.0035</v>
+        <v>0</v>
       </c>
       <c r="O52" t="n">
         <v>0</v>
@@ -4282,7 +4282,7 @@
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>0</v>
+        <v>0.3405</v>
       </c>
       <c r="G53" t="n">
         <v>0</v>
@@ -4291,7 +4291,7 @@
         <v>0</v>
       </c>
       <c r="I53" t="n">
-        <v>0</v>
+        <v>0.0185</v>
       </c>
       <c r="J53" t="n">
         <v>0</v>
@@ -4306,7 +4306,7 @@
         <v>0</v>
       </c>
       <c r="N53" t="n">
-        <v>0.0185</v>
+        <v>0</v>
       </c>
       <c r="O53" t="n">
         <v>0</v>
@@ -4318,7 +4318,7 @@
         <v>0</v>
       </c>
       <c r="R53" t="n">
-        <v>0.3405</v>
+        <v>0</v>
       </c>
       <c r="S53" t="n">
         <v>0</v>
@@ -4361,19 +4361,19 @@
         <v>0</v>
       </c>
       <c r="H54" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" t="n">
         <v>0.0154</v>
-      </c>
-      <c r="I54" t="n">
-        <v>1.2645</v>
-      </c>
-      <c r="J54" t="n">
-        <v>0.0463</v>
-      </c>
-      <c r="K54" t="n">
-        <v>0.0154</v>
-      </c>
-      <c r="L54" t="n">
-        <v>0</v>
       </c>
       <c r="M54" t="n">
         <v>0.3547</v>
@@ -4382,7 +4382,7 @@
         <v>0</v>
       </c>
       <c r="O54" t="n">
-        <v>0</v>
+        <v>0.0154</v>
       </c>
       <c r="P54" t="n">
         <v>0</v>
@@ -4391,22 +4391,22 @@
         <v>0</v>
       </c>
       <c r="R54" t="n">
-        <v>0</v>
+        <v>0.0154</v>
       </c>
       <c r="S54" t="n">
-        <v>0</v>
+        <v>0.0308</v>
       </c>
       <c r="T54" t="n">
-        <v>0.0308</v>
+        <v>0</v>
       </c>
       <c r="U54" t="n">
-        <v>0</v>
+        <v>0.0463</v>
       </c>
       <c r="V54" t="n">
-        <v>0.0154</v>
+        <v>0</v>
       </c>
       <c r="W54" t="n">
-        <v>0</v>
+        <v>1.2645</v>
       </c>
     </row>
     <row r="55">
@@ -4425,7 +4425,7 @@
         <v>0</v>
       </c>
       <c r="E55" t="n">
-        <v>0.0384</v>
+        <v>0</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
@@ -4434,52 +4434,52 @@
         <v>0</v>
       </c>
       <c r="H55" t="n">
+        <v>3.1508</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" t="n">
+        <v>0.1537</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0.1921</v>
+      </c>
+      <c r="L55" t="n">
         <v>2.7089</v>
-      </c>
-      <c r="I55" t="n">
-        <v>1.3641</v>
-      </c>
-      <c r="J55" t="n">
-        <v>0.1153</v>
-      </c>
-      <c r="K55" t="n">
-        <v>8.9337</v>
-      </c>
-      <c r="L55" t="n">
-        <v>0</v>
       </c>
       <c r="M55" t="n">
         <v>0.07679999999999999</v>
       </c>
       <c r="N55" t="n">
-        <v>0</v>
+        <v>0.0384</v>
       </c>
       <c r="O55" t="n">
-        <v>0.1921</v>
+        <v>0</v>
       </c>
       <c r="P55" t="n">
         <v>0</v>
       </c>
       <c r="Q55" t="n">
-        <v>3.1508</v>
+        <v>1.3256</v>
       </c>
       <c r="R55" t="n">
-        <v>0</v>
+        <v>8.9337</v>
       </c>
       <c r="S55" t="n">
-        <v>0</v>
+        <v>0.1537</v>
       </c>
       <c r="T55" t="n">
-        <v>0.1537</v>
+        <v>0</v>
       </c>
       <c r="U55" t="n">
-        <v>1.3256</v>
+        <v>0.1153</v>
       </c>
       <c r="V55" t="n">
         <v>0</v>
       </c>
       <c r="W55" t="n">
-        <v>0.1537</v>
+        <v>1.3641</v>
       </c>
     </row>
     <row r="56">
@@ -4495,64 +4495,64 @@
         <v>1</v>
       </c>
       <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="n">
         <v>0.035</v>
       </c>
-      <c r="E56" t="n">
-        <v>0.1086</v>
-      </c>
       <c r="F56" t="n">
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>0</v>
+        <v>0.0526</v>
       </c>
       <c r="H56" t="n">
+        <v>3.6191</v>
+      </c>
+      <c r="I56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0.1331</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0.1717</v>
+      </c>
+      <c r="L56" t="n">
         <v>3.0515</v>
-      </c>
-      <c r="I56" t="n">
-        <v>1.2613</v>
-      </c>
-      <c r="J56" t="n">
-        <v>0.0385</v>
-      </c>
-      <c r="K56" t="n">
-        <v>10.5735</v>
-      </c>
-      <c r="L56" t="n">
-        <v>0</v>
       </c>
       <c r="M56" t="n">
         <v>0.049</v>
       </c>
       <c r="N56" t="n">
-        <v>0</v>
+        <v>0.1086</v>
       </c>
       <c r="O56" t="n">
-        <v>0.1717</v>
+        <v>0.007</v>
       </c>
       <c r="P56" t="n">
-        <v>0.0526</v>
+        <v>0</v>
       </c>
       <c r="Q56" t="n">
-        <v>3.6191</v>
+        <v>0.9459</v>
       </c>
       <c r="R56" t="n">
-        <v>0</v>
+        <v>10.5735</v>
       </c>
       <c r="S56" t="n">
-        <v>0</v>
+        <v>0.0911</v>
       </c>
       <c r="T56" t="n">
-        <v>0.0911</v>
+        <v>0</v>
       </c>
       <c r="U56" t="n">
-        <v>0.9459</v>
+        <v>0.0385</v>
       </c>
       <c r="V56" t="n">
-        <v>0.007</v>
+        <v>0</v>
       </c>
       <c r="W56" t="n">
-        <v>0.1331</v>
+        <v>1.2613</v>
       </c>
     </row>
     <row r="57">
@@ -4589,7 +4589,7 @@
         <v>0</v>
       </c>
       <c r="K57" t="n">
-        <v>0</v>
+        <v>0.98</v>
       </c>
       <c r="L57" t="n">
         <v>0</v>
@@ -4601,7 +4601,7 @@
         <v>0</v>
       </c>
       <c r="O57" t="n">
-        <v>0.98</v>
+        <v>0</v>
       </c>
       <c r="P57" t="n">
         <v>0</v>
@@ -4641,11 +4641,11 @@
         <v>1</v>
       </c>
       <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="n">
         <v>0.0036</v>
       </c>
-      <c r="E58" t="n">
-        <v>0</v>
-      </c>
       <c r="F58" t="n">
         <v>0</v>
       </c>
@@ -4653,19 +4653,19 @@
         <v>0</v>
       </c>
       <c r="H58" t="n">
+        <v>0.0053</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0.0036</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" t="n">
         <v>0.0338</v>
-      </c>
-      <c r="I58" t="n">
-        <v>0.0587</v>
-      </c>
-      <c r="J58" t="n">
-        <v>0.1174</v>
-      </c>
-      <c r="K58" t="n">
-        <v>0</v>
-      </c>
-      <c r="L58" t="n">
-        <v>0</v>
       </c>
       <c r="M58" t="n">
         <v>4.7884</v>
@@ -4674,31 +4674,31 @@
         <v>0</v>
       </c>
       <c r="O58" t="n">
-        <v>0</v>
+        <v>0.0053</v>
       </c>
       <c r="P58" t="n">
         <v>0</v>
       </c>
       <c r="Q58" t="n">
-        <v>0.0053</v>
+        <v>0</v>
       </c>
       <c r="R58" t="n">
         <v>0</v>
       </c>
       <c r="S58" t="n">
-        <v>0</v>
+        <v>0.0391</v>
       </c>
       <c r="T58" t="n">
-        <v>0.0391</v>
+        <v>0</v>
       </c>
       <c r="U58" t="n">
-        <v>0</v>
+        <v>0.1174</v>
       </c>
       <c r="V58" t="n">
-        <v>0.0053</v>
+        <v>0</v>
       </c>
       <c r="W58" t="n">
-        <v>0.0036</v>
+        <v>0.0587</v>
       </c>
     </row>
     <row r="59">
@@ -4723,52 +4723,52 @@
         <v>0</v>
       </c>
       <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0.1488</v>
+      </c>
+      <c r="L59" t="n">
+        <v>0</v>
+      </c>
+      <c r="M59" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" t="n">
+        <v>0</v>
+      </c>
+      <c r="O59" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>0.2975</v>
+      </c>
+      <c r="R59" t="n">
+        <v>0</v>
+      </c>
+      <c r="S59" t="n">
+        <v>0</v>
+      </c>
+      <c r="T59" t="n">
+        <v>0</v>
+      </c>
+      <c r="U59" t="n">
+        <v>0</v>
+      </c>
+      <c r="V59" t="n">
         <v>0.502</v>
-      </c>
-      <c r="H59" t="n">
-        <v>0</v>
-      </c>
-      <c r="I59" t="n">
-        <v>0</v>
-      </c>
-      <c r="J59" t="n">
-        <v>0</v>
-      </c>
-      <c r="K59" t="n">
-        <v>0</v>
-      </c>
-      <c r="L59" t="n">
-        <v>0</v>
-      </c>
-      <c r="M59" t="n">
-        <v>0</v>
-      </c>
-      <c r="N59" t="n">
-        <v>0</v>
-      </c>
-      <c r="O59" t="n">
-        <v>0.1488</v>
-      </c>
-      <c r="P59" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q59" t="n">
-        <v>0</v>
-      </c>
-      <c r="R59" t="n">
-        <v>0</v>
-      </c>
-      <c r="S59" t="n">
-        <v>0</v>
-      </c>
-      <c r="T59" t="n">
-        <v>0</v>
-      </c>
-      <c r="U59" t="n">
-        <v>0.2975</v>
-      </c>
-      <c r="V59" t="n">
-        <v>0</v>
       </c>
       <c r="W59" t="n">
         <v>0</v>
@@ -4796,19 +4796,19 @@
         <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>0.0218</v>
+        <v>0</v>
       </c>
       <c r="H60" t="n">
         <v>0</v>
       </c>
       <c r="I60" t="n">
-        <v>0</v>
+        <v>0.0044</v>
       </c>
       <c r="J60" t="n">
         <v>0</v>
       </c>
       <c r="K60" t="n">
-        <v>0</v>
+        <v>0.9507</v>
       </c>
       <c r="L60" t="n">
         <v>0</v>
@@ -4817,16 +4817,16 @@
         <v>0.0131</v>
       </c>
       <c r="N60" t="n">
-        <v>0.0044</v>
+        <v>0</v>
       </c>
       <c r="O60" t="n">
-        <v>0.9507</v>
+        <v>0</v>
       </c>
       <c r="P60" t="n">
         <v>0</v>
       </c>
       <c r="Q60" t="n">
-        <v>0</v>
+        <v>1.1426</v>
       </c>
       <c r="R60" t="n">
         <v>0</v>
@@ -4838,10 +4838,10 @@
         <v>0</v>
       </c>
       <c r="U60" t="n">
-        <v>1.1426</v>
+        <v>0</v>
       </c>
       <c r="V60" t="n">
-        <v>0</v>
+        <v>0.0218</v>
       </c>
       <c r="W60" t="n">
         <v>0</v>
@@ -4881,7 +4881,7 @@
         <v>0</v>
       </c>
       <c r="K61" t="n">
-        <v>0</v>
+        <v>0.6935</v>
       </c>
       <c r="L61" t="n">
         <v>0</v>
@@ -4893,13 +4893,13 @@
         <v>0</v>
       </c>
       <c r="O61" t="n">
-        <v>0.6935</v>
+        <v>0</v>
       </c>
       <c r="P61" t="n">
         <v>0</v>
       </c>
       <c r="Q61" t="n">
-        <v>0</v>
+        <v>1.1096</v>
       </c>
       <c r="R61" t="n">
         <v>0</v>
@@ -4911,7 +4911,7 @@
         <v>0</v>
       </c>
       <c r="U61" t="n">
-        <v>1.1096</v>
+        <v>0</v>
       </c>
       <c r="V61" t="n">
         <v>0</v>
@@ -4954,7 +4954,7 @@
         <v>0</v>
       </c>
       <c r="K62" t="n">
-        <v>0</v>
+        <v>2.2</v>
       </c>
       <c r="L62" t="n">
         <v>0</v>
@@ -4966,13 +4966,13 @@
         <v>0</v>
       </c>
       <c r="O62" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
       <c r="P62" t="n">
         <v>0</v>
       </c>
       <c r="Q62" t="n">
-        <v>0</v>
+        <v>7.76</v>
       </c>
       <c r="R62" t="n">
         <v>0</v>
@@ -4984,7 +4984,7 @@
         <v>0</v>
       </c>
       <c r="U62" t="n">
-        <v>7.76</v>
+        <v>0</v>
       </c>
       <c r="V62" t="n">
         <v>0</v>
@@ -5006,7 +5006,7 @@
         <v>2</v>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>0.5444</v>
       </c>
       <c r="E63" t="n">
         <v>0</v>
@@ -5021,7 +5021,7 @@
         <v>0</v>
       </c>
       <c r="I63" t="n">
-        <v>0</v>
+        <v>0.2722</v>
       </c>
       <c r="J63" t="n">
         <v>0</v>
@@ -5030,13 +5030,13 @@
         <v>0</v>
       </c>
       <c r="L63" t="n">
-        <v>0.5444</v>
+        <v>0</v>
       </c>
       <c r="M63" t="n">
         <v>0.4355</v>
       </c>
       <c r="N63" t="n">
-        <v>0.2722</v>
+        <v>0</v>
       </c>
       <c r="O63" t="n">
         <v>0</v>
@@ -5100,7 +5100,7 @@
         <v>0</v>
       </c>
       <c r="K64" t="n">
-        <v>0</v>
+        <v>2.63</v>
       </c>
       <c r="L64" t="n">
         <v>0</v>
@@ -5112,13 +5112,13 @@
         <v>0</v>
       </c>
       <c r="O64" t="n">
-        <v>2.63</v>
+        <v>0</v>
       </c>
       <c r="P64" t="n">
         <v>0</v>
       </c>
       <c r="Q64" t="n">
-        <v>0</v>
+        <v>2.18</v>
       </c>
       <c r="R64" t="n">
         <v>0</v>
@@ -5130,7 +5130,7 @@
         <v>0</v>
       </c>
       <c r="U64" t="n">
-        <v>2.18</v>
+        <v>0</v>
       </c>
       <c r="V64" t="n">
         <v>0</v>
@@ -5234,52 +5234,52 @@
         <v>0</v>
       </c>
       <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" t="n">
+        <v>0</v>
+      </c>
+      <c r="M66" t="n">
+        <v>0</v>
+      </c>
+      <c r="N66" t="n">
+        <v>0</v>
+      </c>
+      <c r="O66" t="n">
+        <v>0</v>
+      </c>
+      <c r="P66" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>0</v>
+      </c>
+      <c r="R66" t="n">
+        <v>0</v>
+      </c>
+      <c r="S66" t="n">
+        <v>0</v>
+      </c>
+      <c r="T66" t="n">
+        <v>0</v>
+      </c>
+      <c r="U66" t="n">
+        <v>0</v>
+      </c>
+      <c r="V66" t="n">
         <v>0.0688</v>
-      </c>
-      <c r="H66" t="n">
-        <v>0</v>
-      </c>
-      <c r="I66" t="n">
-        <v>0</v>
-      </c>
-      <c r="J66" t="n">
-        <v>0</v>
-      </c>
-      <c r="K66" t="n">
-        <v>0</v>
-      </c>
-      <c r="L66" t="n">
-        <v>0</v>
-      </c>
-      <c r="M66" t="n">
-        <v>0</v>
-      </c>
-      <c r="N66" t="n">
-        <v>0</v>
-      </c>
-      <c r="O66" t="n">
-        <v>0</v>
-      </c>
-      <c r="P66" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q66" t="n">
-        <v>0</v>
-      </c>
-      <c r="R66" t="n">
-        <v>0</v>
-      </c>
-      <c r="S66" t="n">
-        <v>0</v>
-      </c>
-      <c r="T66" t="n">
-        <v>0</v>
-      </c>
-      <c r="U66" t="n">
-        <v>0</v>
-      </c>
-      <c r="V66" t="n">
-        <v>0</v>
       </c>
       <c r="W66" t="n">
         <v>0</v>
@@ -5313,49 +5313,49 @@
         <v>0</v>
       </c>
       <c r="I67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" t="n">
+        <v>0</v>
+      </c>
+      <c r="M67" t="n">
+        <v>0</v>
+      </c>
+      <c r="N67" t="n">
+        <v>0</v>
+      </c>
+      <c r="O67" t="n">
+        <v>0</v>
+      </c>
+      <c r="P67" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="R67" t="n">
+        <v>0</v>
+      </c>
+      <c r="S67" t="n">
+        <v>0</v>
+      </c>
+      <c r="T67" t="n">
+        <v>0</v>
+      </c>
+      <c r="U67" t="n">
+        <v>0</v>
+      </c>
+      <c r="V67" t="n">
+        <v>0</v>
+      </c>
+      <c r="W67" t="n">
         <v>5.11</v>
-      </c>
-      <c r="J67" t="n">
-        <v>0</v>
-      </c>
-      <c r="K67" t="n">
-        <v>0</v>
-      </c>
-      <c r="L67" t="n">
-        <v>0</v>
-      </c>
-      <c r="M67" t="n">
-        <v>0</v>
-      </c>
-      <c r="N67" t="n">
-        <v>0</v>
-      </c>
-      <c r="O67" t="n">
-        <v>0</v>
-      </c>
-      <c r="P67" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q67" t="n">
-        <v>0</v>
-      </c>
-      <c r="R67" t="n">
-        <v>0</v>
-      </c>
-      <c r="S67" t="n">
-        <v>0</v>
-      </c>
-      <c r="T67" t="n">
-        <v>0</v>
-      </c>
-      <c r="U67" t="n">
-        <v>5.23</v>
-      </c>
-      <c r="V67" t="n">
-        <v>0</v>
-      </c>
-      <c r="W67" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -5392,7 +5392,7 @@
         <v>0</v>
       </c>
       <c r="K68" t="n">
-        <v>0</v>
+        <v>3.0508</v>
       </c>
       <c r="L68" t="n">
         <v>0</v>
@@ -5404,13 +5404,13 @@
         <v>0</v>
       </c>
       <c r="O68" t="n">
-        <v>3.0508</v>
+        <v>0</v>
       </c>
       <c r="P68" t="n">
         <v>0</v>
       </c>
       <c r="Q68" t="n">
-        <v>0</v>
+        <v>0.2183</v>
       </c>
       <c r="R68" t="n">
         <v>0</v>
@@ -5422,7 +5422,7 @@
         <v>0</v>
       </c>
       <c r="U68" t="n">
-        <v>0.2183</v>
+        <v>0</v>
       </c>
       <c r="V68" t="n">
         <v>0</v>
@@ -5447,61 +5447,61 @@
         <v>0</v>
       </c>
       <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" t="n">
+        <v>0</v>
+      </c>
+      <c r="M69" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" t="n">
         <v>2.3</v>
       </c>
-      <c r="F69" t="n">
-        <v>0</v>
-      </c>
-      <c r="G69" t="n">
-        <v>0</v>
-      </c>
-      <c r="H69" t="n">
-        <v>0</v>
-      </c>
-      <c r="I69" t="n">
+      <c r="O69" t="n">
+        <v>0</v>
+      </c>
+      <c r="P69" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>0</v>
+      </c>
+      <c r="R69" t="n">
+        <v>0</v>
+      </c>
+      <c r="S69" t="n">
+        <v>0</v>
+      </c>
+      <c r="T69" t="n">
+        <v>0</v>
+      </c>
+      <c r="U69" t="n">
+        <v>0</v>
+      </c>
+      <c r="V69" t="n">
+        <v>0</v>
+      </c>
+      <c r="W69" t="n">
         <v>1.25</v>
-      </c>
-      <c r="J69" t="n">
-        <v>0</v>
-      </c>
-      <c r="K69" t="n">
-        <v>0</v>
-      </c>
-      <c r="L69" t="n">
-        <v>0</v>
-      </c>
-      <c r="M69" t="n">
-        <v>0</v>
-      </c>
-      <c r="N69" t="n">
-        <v>0</v>
-      </c>
-      <c r="O69" t="n">
-        <v>0</v>
-      </c>
-      <c r="P69" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q69" t="n">
-        <v>0</v>
-      </c>
-      <c r="R69" t="n">
-        <v>0</v>
-      </c>
-      <c r="S69" t="n">
-        <v>0</v>
-      </c>
-      <c r="T69" t="n">
-        <v>0</v>
-      </c>
-      <c r="U69" t="n">
-        <v>0</v>
-      </c>
-      <c r="V69" t="n">
-        <v>0</v>
-      </c>
-      <c r="W69" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -5526,52 +5526,52 @@
         <v>0</v>
       </c>
       <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" t="n">
+        <v>0</v>
+      </c>
+      <c r="M70" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" t="n">
+        <v>0</v>
+      </c>
+      <c r="O70" t="n">
+        <v>0</v>
+      </c>
+      <c r="P70" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R70" t="n">
+        <v>0</v>
+      </c>
+      <c r="S70" t="n">
+        <v>0</v>
+      </c>
+      <c r="T70" t="n">
+        <v>0</v>
+      </c>
+      <c r="U70" t="n">
+        <v>0</v>
+      </c>
+      <c r="V70" t="n">
         <v>0.72</v>
-      </c>
-      <c r="H70" t="n">
-        <v>0</v>
-      </c>
-      <c r="I70" t="n">
-        <v>0</v>
-      </c>
-      <c r="J70" t="n">
-        <v>0</v>
-      </c>
-      <c r="K70" t="n">
-        <v>0</v>
-      </c>
-      <c r="L70" t="n">
-        <v>0</v>
-      </c>
-      <c r="M70" t="n">
-        <v>0</v>
-      </c>
-      <c r="N70" t="n">
-        <v>0</v>
-      </c>
-      <c r="O70" t="n">
-        <v>0</v>
-      </c>
-      <c r="P70" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q70" t="n">
-        <v>0</v>
-      </c>
-      <c r="R70" t="n">
-        <v>0</v>
-      </c>
-      <c r="S70" t="n">
-        <v>0</v>
-      </c>
-      <c r="T70" t="n">
-        <v>0</v>
-      </c>
-      <c r="U70" t="n">
-        <v>0</v>
-      </c>
-      <c r="V70" t="n">
-        <v>0</v>
       </c>
       <c r="W70" t="n">
         <v>0</v>
@@ -5596,55 +5596,55 @@
         <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>0</v>
+        <v>0.1935</v>
       </c>
       <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0</v>
+      </c>
+      <c r="L71" t="n">
+        <v>0</v>
+      </c>
+      <c r="M71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" t="n">
+        <v>0</v>
+      </c>
+      <c r="O71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>0</v>
+      </c>
+      <c r="R71" t="n">
+        <v>0</v>
+      </c>
+      <c r="S71" t="n">
+        <v>0</v>
+      </c>
+      <c r="T71" t="n">
+        <v>0</v>
+      </c>
+      <c r="U71" t="n">
+        <v>0</v>
+      </c>
+      <c r="V71" t="n">
         <v>0.0506</v>
-      </c>
-      <c r="H71" t="n">
-        <v>0</v>
-      </c>
-      <c r="I71" t="n">
-        <v>0</v>
-      </c>
-      <c r="J71" t="n">
-        <v>0</v>
-      </c>
-      <c r="K71" t="n">
-        <v>0</v>
-      </c>
-      <c r="L71" t="n">
-        <v>0</v>
-      </c>
-      <c r="M71" t="n">
-        <v>0</v>
-      </c>
-      <c r="N71" t="n">
-        <v>0</v>
-      </c>
-      <c r="O71" t="n">
-        <v>0</v>
-      </c>
-      <c r="P71" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q71" t="n">
-        <v>0</v>
-      </c>
-      <c r="R71" t="n">
-        <v>0.1935</v>
-      </c>
-      <c r="S71" t="n">
-        <v>0</v>
-      </c>
-      <c r="T71" t="n">
-        <v>0</v>
-      </c>
-      <c r="U71" t="n">
-        <v>0</v>
-      </c>
-      <c r="V71" t="n">
-        <v>0</v>
       </c>
       <c r="W71" t="n">
         <v>0</v>

</xml_diff>